<commit_message>
Updated coverage_report.xlsx for sprint 1
</commit_message>
<xml_diff>
--- a/Evidence/MA/coverage_report.xlsx
+++ b/Evidence/MA/coverage_report.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raygu\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raygu\Downloads\CO3095-Group-16-Music-Player-Application\Evidence\MA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8D087A2F-2C48-4D4F-9C02-8D8B16787F50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57DAF4F1-C8A5-4682-B970-39B4BEA05ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{B4F26AE1-5879-47D9-8144-9A3C1A46093E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="54">
   <si>
     <t>Story ID</t>
   </si>
@@ -74,17 +74,137 @@
     <t>Defects Resolved</t>
   </si>
   <si>
-    <t>Coverage vs Prev Sprint (%)</t>
-  </si>
-  <si>
     <t>Date</t>
+  </si>
+  <si>
+    <t>S1-01</t>
+  </si>
+  <si>
+    <t>S1-02</t>
+  </si>
+  <si>
+    <t>S1-03</t>
+  </si>
+  <si>
+    <t>S1-04</t>
+  </si>
+  <si>
+    <t>S1-05</t>
+  </si>
+  <si>
+    <t>S1-06</t>
+  </si>
+  <si>
+    <t>S1-07</t>
+  </si>
+  <si>
+    <t>S1-08</t>
+  </si>
+  <si>
+    <t>S1-09</t>
+  </si>
+  <si>
+    <t>S1-10</t>
+  </si>
+  <si>
+    <t>S1-11</t>
+  </si>
+  <si>
+    <t>S1-12</t>
+  </si>
+  <si>
+    <t>play/pause/stop</t>
+  </si>
+  <si>
+    <t>blackbox specification</t>
+  </si>
+  <si>
+    <t>blackbox random</t>
+  </si>
+  <si>
+    <t>whitebox</t>
+  </si>
+  <si>
+    <t>next/prev</t>
+  </si>
+  <si>
+    <t>song info</t>
+  </si>
+  <si>
+    <t>volume</t>
+  </si>
+  <si>
+    <t>progress/total time</t>
+  </si>
+  <si>
+    <t>Code Module</t>
+  </si>
+  <si>
+    <t>player_core, player_state</t>
+  </si>
+  <si>
+    <t>player_queue</t>
+  </si>
+  <si>
+    <t>player_ui</t>
+  </si>
+  <si>
+    <t>player_audio</t>
+  </si>
+  <si>
+    <t>progress bar/seek</t>
+  </si>
+  <si>
+    <t>player_ui, player_seek</t>
+  </si>
+  <si>
+    <t>shortcuts</t>
+  </si>
+  <si>
+    <t>player_shortcuts</t>
+  </si>
+  <si>
+    <t>rw/ff</t>
+  </si>
+  <si>
+    <t>player_seek</t>
+  </si>
+  <si>
+    <t>mute</t>
+  </si>
+  <si>
+    <t>indicator</t>
+  </si>
+  <si>
+    <t>help commands</t>
+  </si>
+  <si>
+    <t>player_help</t>
+  </si>
+  <si>
+    <t>background</t>
+  </si>
+  <si>
+    <t>player_core</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Sprint 1 Total Coverage</t>
+  </si>
+  <si>
+    <t>player_core, player_state, player_ui, player_seek, player_shortcuts, player_help, player_audio, player_queue</t>
+  </si>
+  <si>
+    <t>All</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -96,6 +216,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -121,9 +247,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -458,11 +585,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6C833DE-F332-4BAA-A701-CCE6281E1DB6}">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="17.85546875" customWidth="1"/>
-    <col min="4" max="5" width="10.140625" customWidth="1"/>
+    <col min="3" max="3" width="21.28515625" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" customWidth="1"/>
     <col min="6" max="6" width="13.28515625" customWidth="1"/>
     <col min="7" max="7" width="13.42578125" customWidth="1"/>
     <col min="8" max="8" width="14.42578125" customWidth="1"/>
@@ -470,8 +598,8 @@
     <col min="10" max="10" width="13.7109375" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
     <col min="12" max="12" width="17.42578125" customWidth="1"/>
-    <col min="13" max="13" width="31.5703125" customWidth="1"/>
-    <col min="14" max="14" width="15.7109375" customWidth="1"/>
+    <col min="13" max="13" width="15.7109375" customWidth="1"/>
+    <col min="14" max="14" width="96.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -515,10 +643,1639 @@
         <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>13</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2">
+        <v>8</v>
+      </c>
+      <c r="F2">
+        <v>8</v>
+      </c>
+      <c r="G2">
+        <v>100</v>
+      </c>
+      <c r="H2">
+        <v>59</v>
+      </c>
+      <c r="I2">
+        <v>72</v>
+      </c>
+      <c r="J2">
+        <v>82</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3">
+        <v>15</v>
+      </c>
+      <c r="F3">
+        <v>15</v>
+      </c>
+      <c r="G3">
+        <v>100</v>
+      </c>
+      <c r="H3">
+        <v>44</v>
+      </c>
+      <c r="I3">
+        <v>72</v>
+      </c>
+      <c r="J3">
+        <v>61</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4">
+        <v>27</v>
+      </c>
+      <c r="F4">
+        <v>27</v>
+      </c>
+      <c r="G4">
+        <v>100</v>
+      </c>
+      <c r="H4">
+        <v>72</v>
+      </c>
+      <c r="I4">
+        <v>72</v>
+      </c>
+      <c r="J4">
+        <v>100</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5">
+        <v>24</v>
+      </c>
+      <c r="F5">
+        <v>24</v>
+      </c>
+      <c r="G5">
+        <v>100</v>
+      </c>
+      <c r="H5">
+        <v>120</v>
+      </c>
+      <c r="I5">
+        <v>161</v>
+      </c>
+      <c r="J5">
+        <v>75</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6">
+        <v>11</v>
+      </c>
+      <c r="F6">
+        <v>11</v>
+      </c>
+      <c r="G6">
+        <v>100</v>
+      </c>
+      <c r="H6">
+        <v>59</v>
+      </c>
+      <c r="I6">
+        <v>161</v>
+      </c>
+      <c r="J6">
+        <v>37</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7">
+        <v>12</v>
+      </c>
+      <c r="F7">
+        <v>12</v>
+      </c>
+      <c r="G7">
+        <v>100</v>
+      </c>
+      <c r="H7">
+        <v>73</v>
+      </c>
+      <c r="I7">
+        <v>161</v>
+      </c>
+      <c r="J7">
+        <v>45</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8">
+        <v>14</v>
+      </c>
+      <c r="F8">
+        <v>14</v>
+      </c>
+      <c r="G8">
+        <v>100</v>
+      </c>
+      <c r="H8">
+        <v>46</v>
+      </c>
+      <c r="I8">
+        <v>66</v>
+      </c>
+      <c r="J8">
+        <v>70</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9">
+        <v>7</v>
+      </c>
+      <c r="F9">
+        <v>7</v>
+      </c>
+      <c r="G9">
+        <v>100</v>
+      </c>
+      <c r="H9">
+        <v>34</v>
+      </c>
+      <c r="I9">
+        <v>66</v>
+      </c>
+      <c r="J9">
+        <v>52</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10">
+        <v>10</v>
+      </c>
+      <c r="F10">
+        <v>10</v>
+      </c>
+      <c r="G10">
+        <v>100</v>
+      </c>
+      <c r="H10">
+        <v>54</v>
+      </c>
+      <c r="I10">
+        <v>66</v>
+      </c>
+      <c r="J10">
+        <v>82</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11">
+        <v>21</v>
+      </c>
+      <c r="F11">
+        <v>21</v>
+      </c>
+      <c r="G11">
+        <v>100</v>
+      </c>
+      <c r="H11">
+        <v>16</v>
+      </c>
+      <c r="I11">
+        <v>55</v>
+      </c>
+      <c r="J11">
+        <v>29</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12">
+        <v>14</v>
+      </c>
+      <c r="F12">
+        <v>14</v>
+      </c>
+      <c r="G12">
+        <v>100</v>
+      </c>
+      <c r="H12">
+        <v>32</v>
+      </c>
+      <c r="I12">
+        <v>55</v>
+      </c>
+      <c r="J12">
+        <v>58</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13">
+        <v>8</v>
+      </c>
+      <c r="F13">
+        <v>8</v>
+      </c>
+      <c r="G13">
+        <v>100</v>
+      </c>
+      <c r="H13">
+        <v>24</v>
+      </c>
+      <c r="I13">
+        <v>55</v>
+      </c>
+      <c r="J13">
+        <v>44</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N13" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14">
+        <v>21</v>
+      </c>
+      <c r="F14">
+        <v>21</v>
+      </c>
+      <c r="G14">
+        <v>100</v>
+      </c>
+      <c r="H14">
+        <v>25</v>
+      </c>
+      <c r="I14">
+        <v>66</v>
+      </c>
+      <c r="J14">
+        <v>38</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15">
+        <v>7</v>
+      </c>
+      <c r="F15">
+        <v>7</v>
+      </c>
+      <c r="G15">
+        <v>100</v>
+      </c>
+      <c r="H15">
+        <v>34</v>
+      </c>
+      <c r="I15">
+        <v>66</v>
+      </c>
+      <c r="J15">
+        <v>52</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16">
+        <v>8</v>
+      </c>
+      <c r="F16">
+        <v>8</v>
+      </c>
+      <c r="G16">
+        <v>100</v>
+      </c>
+      <c r="H16">
+        <v>35</v>
+      </c>
+      <c r="I16">
+        <v>66</v>
+      </c>
+      <c r="J16">
+        <v>53</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N16" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17">
+        <v>21</v>
+      </c>
+      <c r="F17">
+        <v>21</v>
+      </c>
+      <c r="G17">
+        <v>100</v>
+      </c>
+      <c r="H17">
+        <v>58</v>
+      </c>
+      <c r="I17">
+        <v>101</v>
+      </c>
+      <c r="J17">
+        <v>57</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N17" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18">
+        <v>26</v>
+      </c>
+      <c r="F18">
+        <v>26</v>
+      </c>
+      <c r="G18">
+        <v>100</v>
+      </c>
+      <c r="H18">
+        <v>54</v>
+      </c>
+      <c r="I18">
+        <v>101</v>
+      </c>
+      <c r="J18">
+        <v>53</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N18" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
+        <v>38</v>
+      </c>
+      <c r="D19" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19">
+        <v>21</v>
+      </c>
+      <c r="F19">
+        <v>21</v>
+      </c>
+      <c r="G19">
+        <v>100</v>
+      </c>
+      <c r="H19">
+        <v>61</v>
+      </c>
+      <c r="I19">
+        <v>101</v>
+      </c>
+      <c r="J19">
+        <v>60</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N19" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
+        <v>40</v>
+      </c>
+      <c r="D20" t="s">
+        <v>26</v>
+      </c>
+      <c r="E20">
+        <v>7</v>
+      </c>
+      <c r="F20">
+        <v>7</v>
+      </c>
+      <c r="G20">
+        <v>100</v>
+      </c>
+      <c r="H20">
+        <v>13</v>
+      </c>
+      <c r="I20">
+        <v>13</v>
+      </c>
+      <c r="J20">
+        <v>100</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>0</v>
+      </c>
+      <c r="M20" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N20" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21">
+        <v>4</v>
+      </c>
+      <c r="F21">
+        <v>4</v>
+      </c>
+      <c r="G21">
+        <v>100</v>
+      </c>
+      <c r="H21">
+        <v>8</v>
+      </c>
+      <c r="I21">
+        <v>13</v>
+      </c>
+      <c r="J21">
+        <v>62</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="L21">
+        <v>0</v>
+      </c>
+      <c r="M21" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N21" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
+        <v>40</v>
+      </c>
+      <c r="D22" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22">
+        <v>9</v>
+      </c>
+      <c r="F22">
+        <v>9</v>
+      </c>
+      <c r="G22">
+        <v>100</v>
+      </c>
+      <c r="H22">
+        <v>13</v>
+      </c>
+      <c r="I22">
+        <v>13</v>
+      </c>
+      <c r="J22">
+        <v>100</v>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+      <c r="L22">
+        <v>0</v>
+      </c>
+      <c r="M22" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N22" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>42</v>
+      </c>
+      <c r="D23" t="s">
+        <v>26</v>
+      </c>
+      <c r="E23">
+        <v>7</v>
+      </c>
+      <c r="F23">
+        <v>7</v>
+      </c>
+      <c r="G23">
+        <v>100</v>
+      </c>
+      <c r="H23">
+        <v>19</v>
+      </c>
+      <c r="I23">
+        <v>35</v>
+      </c>
+      <c r="J23">
+        <v>54</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="L23">
+        <v>0</v>
+      </c>
+      <c r="M23" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N23" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" t="s">
+        <v>27</v>
+      </c>
+      <c r="E24">
+        <v>6</v>
+      </c>
+      <c r="F24">
+        <v>6</v>
+      </c>
+      <c r="G24">
+        <v>100</v>
+      </c>
+      <c r="H24">
+        <v>20</v>
+      </c>
+      <c r="I24">
+        <v>35</v>
+      </c>
+      <c r="J24">
+        <v>57</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+      <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N24" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>20</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+      <c r="C25" t="s">
+        <v>42</v>
+      </c>
+      <c r="D25" t="s">
+        <v>28</v>
+      </c>
+      <c r="E25">
+        <v>13</v>
+      </c>
+      <c r="F25">
+        <v>13</v>
+      </c>
+      <c r="G25">
+        <v>100</v>
+      </c>
+      <c r="H25">
+        <v>26</v>
+      </c>
+      <c r="I25">
+        <v>35</v>
+      </c>
+      <c r="J25">
+        <v>74</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+      <c r="L25">
+        <v>0</v>
+      </c>
+      <c r="M25" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N25" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>21</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26" t="s">
+        <v>44</v>
+      </c>
+      <c r="D26" t="s">
+        <v>26</v>
+      </c>
+      <c r="E26">
+        <v>24</v>
+      </c>
+      <c r="F26">
+        <v>24</v>
+      </c>
+      <c r="G26">
+        <v>100</v>
+      </c>
+      <c r="H26">
+        <v>16</v>
+      </c>
+      <c r="I26">
+        <v>55</v>
+      </c>
+      <c r="J26">
+        <v>29</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+      <c r="L26">
+        <v>0</v>
+      </c>
+      <c r="M26" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N26" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>21</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>44</v>
+      </c>
+      <c r="D27" t="s">
+        <v>27</v>
+      </c>
+      <c r="E27">
+        <v>14</v>
+      </c>
+      <c r="F27">
+        <v>14</v>
+      </c>
+      <c r="G27">
+        <v>100</v>
+      </c>
+      <c r="H27">
+        <v>32</v>
+      </c>
+      <c r="I27">
+        <v>55</v>
+      </c>
+      <c r="J27">
+        <v>58</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27">
+        <v>0</v>
+      </c>
+      <c r="M27" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N27" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>21</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28" t="s">
+        <v>44</v>
+      </c>
+      <c r="D28" t="s">
+        <v>28</v>
+      </c>
+      <c r="E28">
+        <v>13</v>
+      </c>
+      <c r="F28">
+        <v>13</v>
+      </c>
+      <c r="G28">
+        <v>100</v>
+      </c>
+      <c r="H28">
+        <v>34</v>
+      </c>
+      <c r="I28">
+        <v>55</v>
+      </c>
+      <c r="J28">
+        <v>62</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+      <c r="L28">
+        <v>0</v>
+      </c>
+      <c r="M28" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N28" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>22</v>
+      </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+      <c r="C29" t="s">
+        <v>45</v>
+      </c>
+      <c r="D29" t="s">
+        <v>26</v>
+      </c>
+      <c r="E29">
+        <v>14</v>
+      </c>
+      <c r="F29">
+        <v>14</v>
+      </c>
+      <c r="G29">
+        <v>100</v>
+      </c>
+      <c r="H29">
+        <v>46</v>
+      </c>
+      <c r="I29">
+        <v>66</v>
+      </c>
+      <c r="J29">
+        <v>70</v>
+      </c>
+      <c r="K29">
+        <v>0</v>
+      </c>
+      <c r="L29">
+        <v>0</v>
+      </c>
+      <c r="M29" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N29" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>22</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30" t="s">
+        <v>45</v>
+      </c>
+      <c r="D30" t="s">
+        <v>27</v>
+      </c>
+      <c r="E30">
+        <v>7</v>
+      </c>
+      <c r="F30">
+        <v>7</v>
+      </c>
+      <c r="G30">
+        <v>100</v>
+      </c>
+      <c r="H30">
+        <v>34</v>
+      </c>
+      <c r="I30">
+        <v>66</v>
+      </c>
+      <c r="J30">
+        <v>52</v>
+      </c>
+      <c r="K30">
+        <v>0</v>
+      </c>
+      <c r="L30">
+        <v>0</v>
+      </c>
+      <c r="M30" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N30" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>22</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>45</v>
+      </c>
+      <c r="D31" t="s">
+        <v>28</v>
+      </c>
+      <c r="E31">
+        <v>10</v>
+      </c>
+      <c r="F31">
+        <v>10</v>
+      </c>
+      <c r="G31">
+        <v>100</v>
+      </c>
+      <c r="H31">
+        <v>54</v>
+      </c>
+      <c r="I31">
+        <v>66</v>
+      </c>
+      <c r="J31">
+        <v>82</v>
+      </c>
+      <c r="K31">
+        <v>0</v>
+      </c>
+      <c r="L31">
+        <v>0</v>
+      </c>
+      <c r="M31" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N31" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>23</v>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>46</v>
+      </c>
+      <c r="D32" t="s">
+        <v>26</v>
+      </c>
+      <c r="E32">
+        <v>24</v>
+      </c>
+      <c r="F32">
+        <v>24</v>
+      </c>
+      <c r="G32">
+        <v>100</v>
+      </c>
+      <c r="H32">
+        <v>37</v>
+      </c>
+      <c r="I32">
+        <v>79</v>
+      </c>
+      <c r="J32">
+        <v>47</v>
+      </c>
+      <c r="K32">
+        <v>0</v>
+      </c>
+      <c r="L32">
+        <v>0</v>
+      </c>
+      <c r="M32" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N32" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>23</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
+        <v>46</v>
+      </c>
+      <c r="D33" t="s">
+        <v>27</v>
+      </c>
+      <c r="E33">
+        <v>18</v>
+      </c>
+      <c r="F33">
+        <v>18</v>
+      </c>
+      <c r="G33">
+        <v>100</v>
+      </c>
+      <c r="H33">
+        <v>52</v>
+      </c>
+      <c r="I33">
+        <v>79</v>
+      </c>
+      <c r="J33">
+        <v>66</v>
+      </c>
+      <c r="K33">
+        <v>0</v>
+      </c>
+      <c r="L33">
+        <v>0</v>
+      </c>
+      <c r="M33" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N33" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>23</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>46</v>
+      </c>
+      <c r="D34" t="s">
+        <v>28</v>
+      </c>
+      <c r="E34">
+        <v>20</v>
+      </c>
+      <c r="F34">
+        <v>20</v>
+      </c>
+      <c r="G34">
+        <v>100</v>
+      </c>
+      <c r="H34">
+        <v>70</v>
+      </c>
+      <c r="I34">
+        <v>79</v>
+      </c>
+      <c r="J34">
+        <v>89</v>
+      </c>
+      <c r="K34">
+        <v>0</v>
+      </c>
+      <c r="L34">
+        <v>0</v>
+      </c>
+      <c r="M34" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N34" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>24</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>48</v>
+      </c>
+      <c r="D35" t="s">
+        <v>26</v>
+      </c>
+      <c r="E35">
+        <v>14</v>
+      </c>
+      <c r="F35">
+        <v>14</v>
+      </c>
+      <c r="G35">
+        <v>100</v>
+      </c>
+      <c r="H35">
+        <v>38</v>
+      </c>
+      <c r="I35">
+        <v>50</v>
+      </c>
+      <c r="J35">
+        <v>76</v>
+      </c>
+      <c r="K35">
+        <v>0</v>
+      </c>
+      <c r="L35">
+        <v>0</v>
+      </c>
+      <c r="M35" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N35" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>24</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+      <c r="C36" t="s">
+        <v>48</v>
+      </c>
+      <c r="D36" t="s">
+        <v>27</v>
+      </c>
+      <c r="E36">
+        <v>7</v>
+      </c>
+      <c r="F36">
+        <v>7</v>
+      </c>
+      <c r="G36">
+        <v>100</v>
+      </c>
+      <c r="H36">
+        <v>23</v>
+      </c>
+      <c r="I36">
+        <v>50</v>
+      </c>
+      <c r="J36">
+        <v>46</v>
+      </c>
+      <c r="K36">
+        <v>0</v>
+      </c>
+      <c r="L36">
+        <v>0</v>
+      </c>
+      <c r="M36" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N36" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37" t="s">
+        <v>48</v>
+      </c>
+      <c r="D37" t="s">
+        <v>28</v>
+      </c>
+      <c r="E37">
+        <v>27</v>
+      </c>
+      <c r="F37">
+        <v>27</v>
+      </c>
+      <c r="G37">
+        <v>100</v>
+      </c>
+      <c r="H37">
+        <v>50</v>
+      </c>
+      <c r="I37">
+        <v>50</v>
+      </c>
+      <c r="J37">
+        <v>100</v>
+      </c>
+      <c r="K37">
+        <v>0</v>
+      </c>
+      <c r="L37">
+        <v>0</v>
+      </c>
+      <c r="M37" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N37" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>50</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>51</v>
+      </c>
+      <c r="D38" t="s">
+        <v>53</v>
+      </c>
+      <c r="E38">
+        <v>283</v>
+      </c>
+      <c r="F38">
+        <v>283</v>
+      </c>
+      <c r="G38">
+        <v>100</v>
+      </c>
+      <c r="H38">
+        <v>469</v>
+      </c>
+      <c r="I38">
+        <v>512</v>
+      </c>
+      <c r="J38">
+        <v>92</v>
+      </c>
+      <c r="K38">
+        <v>0</v>
+      </c>
+      <c r="L38">
+        <v>0</v>
+      </c>
+      <c r="M38" s="2">
+        <v>45993</v>
+      </c>
+      <c r="N38" t="s">
+        <v>52</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated coverage_report.xlsx for Sprint 2
</commit_message>
<xml_diff>
--- a/Evidence/MA/coverage_report.xlsx
+++ b/Evidence/MA/coverage_report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raygu\Downloads\CO3095-Group-16-Music-Player-Application\Evidence\MA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raygu\Downloads\CO3095\Evidence\MA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57DAF4F1-C8A5-4682-B970-39B4BEA05ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B83393EE-DEBA-4895-9F07-DD0B2AB4E5E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{B4F26AE1-5879-47D9-8144-9A3C1A46093E}"/>
+    <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="16186" xr2:uid="{B4F26AE1-5879-47D9-8144-9A3C1A46093E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="83">
   <si>
     <t>Story ID</t>
   </si>
@@ -68,12 +68,6 @@
     <t>Coverage (%)</t>
   </si>
   <si>
-    <t>Defects Found</t>
-  </si>
-  <si>
-    <t>Defects Resolved</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
@@ -198,6 +192,99 @@
   </si>
   <si>
     <t>All</t>
+  </si>
+  <si>
+    <t>S2-01</t>
+  </si>
+  <si>
+    <t>S2-02</t>
+  </si>
+  <si>
+    <t>S2-03</t>
+  </si>
+  <si>
+    <t>S2-04</t>
+  </si>
+  <si>
+    <t>S2-05</t>
+  </si>
+  <si>
+    <t>S2-06</t>
+  </si>
+  <si>
+    <t>S2-07</t>
+  </si>
+  <si>
+    <t>S2-08</t>
+  </si>
+  <si>
+    <t>S2-09</t>
+  </si>
+  <si>
+    <t>S2-10</t>
+  </si>
+  <si>
+    <t>S2-11</t>
+  </si>
+  <si>
+    <t>S2-12</t>
+  </si>
+  <si>
+    <t>Sprint 2 Total Coverage</t>
+  </si>
+  <si>
+    <t>create/rename/delete playlists</t>
+  </si>
+  <si>
+    <t>add/remove songs in playlists</t>
+  </si>
+  <si>
+    <t>search songs by title, album, artist</t>
+  </si>
+  <si>
+    <t>view songs in table</t>
+  </si>
+  <si>
+    <t>playlist list</t>
+  </si>
+  <si>
+    <t>open playlist</t>
+  </si>
+  <si>
+    <t>add song with text command</t>
+  </si>
+  <si>
+    <t>add song confirmation message</t>
+  </si>
+  <si>
+    <t>scan main library files</t>
+  </si>
+  <si>
+    <t>playlist number songs and playtime</t>
+  </si>
+  <si>
+    <t>merge playlists</t>
+  </si>
+  <si>
+    <t>copy playlists</t>
+  </si>
+  <si>
+    <t>playlist_model, playlists_basic</t>
+  </si>
+  <si>
+    <t>playlists_edit</t>
+  </si>
+  <si>
+    <t>playlists_advanced</t>
+  </si>
+  <si>
+    <t>library_search_scan</t>
+  </si>
+  <si>
+    <t>playlists_basic</t>
+  </si>
+  <si>
+    <t>playlist_model, playlists_basic, playlists_edit, playlists_advanced, library_search_scan</t>
   </si>
 </sst>
 </file>
@@ -585,24 +672,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6C833DE-F332-4BAA-A701-CCE6281E1DB6}">
-  <dimension ref="A1:N38"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L75"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="3" max="3" width="21.28515625" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" customWidth="1"/>
-    <col min="6" max="6" width="13.28515625" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" customWidth="1"/>
-    <col min="8" max="8" width="14.42578125" customWidth="1"/>
-    <col min="9" max="9" width="10.5703125" customWidth="1"/>
-    <col min="10" max="10" width="13.7109375" customWidth="1"/>
-    <col min="11" max="11" width="15" customWidth="1"/>
-    <col min="12" max="12" width="17.42578125" customWidth="1"/>
-    <col min="13" max="13" width="15.7109375" customWidth="1"/>
-    <col min="14" max="14" width="96.85546875" customWidth="1"/>
+    <col min="3" max="3" width="29.52734375" customWidth="1"/>
+    <col min="4" max="4" width="20.703125" customWidth="1"/>
+    <col min="5" max="5" width="10.1171875" customWidth="1"/>
+    <col min="6" max="6" width="13.29296875" customWidth="1"/>
+    <col min="7" max="7" width="13.41015625" customWidth="1"/>
+    <col min="8" max="8" width="14.41015625" customWidth="1"/>
+    <col min="9" max="9" width="10.5859375" customWidth="1"/>
+    <col min="10" max="10" width="13.703125" customWidth="1"/>
+    <col min="11" max="11" width="15.703125" customWidth="1"/>
+    <col min="12" max="12" width="96.87890625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -637,27 +722,21 @@
         <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E2">
         <v>8</v>
@@ -677,31 +756,25 @@
       <c r="J2">
         <v>82</v>
       </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K2" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
         <v>25</v>
-      </c>
-      <c r="D3" t="s">
-        <v>27</v>
       </c>
       <c r="E3">
         <v>15</v>
@@ -721,31 +794,25 @@
       <c r="J3">
         <v>61</v>
       </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
-      <c r="L3">
-        <v>0</v>
-      </c>
-      <c r="M3" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K3" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E4">
         <v>27</v>
@@ -765,31 +832,25 @@
       <c r="J4">
         <v>100</v>
       </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K4" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E5">
         <v>24</v>
@@ -809,31 +870,25 @@
       <c r="J5">
         <v>75</v>
       </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
-      <c r="L5">
-        <v>0</v>
-      </c>
-      <c r="M5" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K5" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E6">
         <v>11</v>
@@ -853,31 +908,25 @@
       <c r="J6">
         <v>37</v>
       </c>
-      <c r="K6">
-        <v>0</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K6" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E7">
         <v>12</v>
@@ -897,31 +946,25 @@
       <c r="J7">
         <v>45</v>
       </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N7" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K7" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E8">
         <v>14</v>
@@ -941,31 +984,25 @@
       <c r="J8">
         <v>70</v>
       </c>
-      <c r="K8">
-        <v>0</v>
-      </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K8" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E9">
         <v>7</v>
@@ -985,31 +1022,25 @@
       <c r="J9">
         <v>52</v>
       </c>
-      <c r="K9">
-        <v>0</v>
-      </c>
-      <c r="L9">
-        <v>0</v>
-      </c>
-      <c r="M9" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K9" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E10">
         <v>10</v>
@@ -1029,31 +1060,25 @@
       <c r="J10">
         <v>82</v>
       </c>
-      <c r="K10">
-        <v>0</v>
-      </c>
-      <c r="L10">
-        <v>0</v>
-      </c>
-      <c r="M10" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K10" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E11">
         <v>21</v>
@@ -1073,31 +1098,25 @@
       <c r="J11">
         <v>29</v>
       </c>
-      <c r="K11">
-        <v>0</v>
-      </c>
-      <c r="L11">
-        <v>0</v>
-      </c>
-      <c r="M11" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N11" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K11" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B12">
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E12">
         <v>14</v>
@@ -1117,31 +1136,25 @@
       <c r="J12">
         <v>58</v>
       </c>
-      <c r="K12">
-        <v>0</v>
-      </c>
-      <c r="L12">
-        <v>0</v>
-      </c>
-      <c r="M12" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N12" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K12" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E13">
         <v>8</v>
@@ -1161,31 +1174,25 @@
       <c r="J13">
         <v>44</v>
       </c>
-      <c r="K13">
-        <v>0</v>
-      </c>
-      <c r="L13">
-        <v>0</v>
-      </c>
-      <c r="M13" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N13" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K13" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D14" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E14">
         <v>21</v>
@@ -1205,31 +1212,25 @@
       <c r="J14">
         <v>38</v>
       </c>
-      <c r="K14">
-        <v>0</v>
-      </c>
-      <c r="L14">
-        <v>0</v>
-      </c>
-      <c r="M14" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N14" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K14" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E15">
         <v>7</v>
@@ -1249,31 +1250,25 @@
       <c r="J15">
         <v>52</v>
       </c>
-      <c r="K15">
-        <v>0</v>
-      </c>
-      <c r="L15">
-        <v>0</v>
-      </c>
-      <c r="M15" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N15" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K15" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L15" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D16" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E16">
         <v>8</v>
@@ -1293,31 +1288,25 @@
       <c r="J16">
         <v>53</v>
       </c>
-      <c r="K16">
-        <v>0</v>
-      </c>
-      <c r="L16">
-        <v>0</v>
-      </c>
-      <c r="M16" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N16" t="s">
+      <c r="K16" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17">
-        <v>1</v>
-      </c>
-      <c r="C17" t="s">
-        <v>38</v>
-      </c>
       <c r="D17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E17">
         <v>21</v>
@@ -1337,31 +1326,25 @@
       <c r="J17">
         <v>57</v>
       </c>
-      <c r="K17">
-        <v>0</v>
-      </c>
-      <c r="L17">
-        <v>0</v>
-      </c>
-      <c r="M17" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K17" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L17" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B18">
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D18" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E18">
         <v>26</v>
@@ -1381,31 +1364,25 @@
       <c r="J18">
         <v>53</v>
       </c>
-      <c r="K18">
-        <v>0</v>
-      </c>
-      <c r="L18">
-        <v>0</v>
-      </c>
-      <c r="M18" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K18" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L18" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E19">
         <v>21</v>
@@ -1425,31 +1402,25 @@
       <c r="J19">
         <v>60</v>
       </c>
-      <c r="K19">
-        <v>0</v>
-      </c>
-      <c r="L19">
-        <v>0</v>
-      </c>
-      <c r="M19" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N19" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K19" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B20">
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D20" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E20">
         <v>7</v>
@@ -1469,31 +1440,25 @@
       <c r="J20">
         <v>100</v>
       </c>
-      <c r="K20">
-        <v>0</v>
-      </c>
-      <c r="L20">
-        <v>0</v>
-      </c>
-      <c r="M20" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N20" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K20" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L20" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B21">
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D21" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E21">
         <v>4</v>
@@ -1513,31 +1478,25 @@
       <c r="J21">
         <v>62</v>
       </c>
-      <c r="K21">
-        <v>0</v>
-      </c>
-      <c r="L21">
-        <v>0</v>
-      </c>
-      <c r="M21" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N21" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K21" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A22" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B22">
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E22">
         <v>9</v>
@@ -1557,31 +1516,25 @@
       <c r="J22">
         <v>100</v>
       </c>
-      <c r="K22">
-        <v>0</v>
-      </c>
-      <c r="L22">
-        <v>0</v>
-      </c>
-      <c r="M22" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N22" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K22" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A23" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B23">
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D23" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E23">
         <v>7</v>
@@ -1601,31 +1554,25 @@
       <c r="J23">
         <v>54</v>
       </c>
-      <c r="K23">
-        <v>0</v>
-      </c>
-      <c r="L23">
-        <v>0</v>
-      </c>
-      <c r="M23" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N23" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K23" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L23" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A24" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B24">
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D24" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E24">
         <v>6</v>
@@ -1645,31 +1592,25 @@
       <c r="J24">
         <v>57</v>
       </c>
-      <c r="K24">
-        <v>0</v>
-      </c>
-      <c r="L24">
-        <v>0</v>
-      </c>
-      <c r="M24" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N24" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K24" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L24" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A25" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B25">
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D25" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E25">
         <v>13</v>
@@ -1689,31 +1630,25 @@
       <c r="J25">
         <v>74</v>
       </c>
-      <c r="K25">
-        <v>0</v>
-      </c>
-      <c r="L25">
-        <v>0</v>
-      </c>
-      <c r="M25" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N25" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K25" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L25" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A26" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B26">
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D26" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E26">
         <v>24</v>
@@ -1733,31 +1668,25 @@
       <c r="J26">
         <v>29</v>
       </c>
-      <c r="K26">
-        <v>0</v>
-      </c>
-      <c r="L26">
-        <v>0</v>
-      </c>
-      <c r="M26" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N26" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K26" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L26" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A27" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B27">
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D27" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E27">
         <v>14</v>
@@ -1777,31 +1706,25 @@
       <c r="J27">
         <v>58</v>
       </c>
-      <c r="K27">
-        <v>0</v>
-      </c>
-      <c r="L27">
-        <v>0</v>
-      </c>
-      <c r="M27" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N27" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K27" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L27" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A28" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B28">
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D28" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E28">
         <v>13</v>
@@ -1821,31 +1744,25 @@
       <c r="J28">
         <v>62</v>
       </c>
-      <c r="K28">
-        <v>0</v>
-      </c>
-      <c r="L28">
-        <v>0</v>
-      </c>
-      <c r="M28" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N28" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K28" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L28" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A29" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B29">
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D29" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E29">
         <v>14</v>
@@ -1865,31 +1782,25 @@
       <c r="J29">
         <v>70</v>
       </c>
-      <c r="K29">
-        <v>0</v>
-      </c>
-      <c r="L29">
-        <v>0</v>
-      </c>
-      <c r="M29" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N29" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K29" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L29" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A30" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B30">
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D30" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E30">
         <v>7</v>
@@ -1909,31 +1820,25 @@
       <c r="J30">
         <v>52</v>
       </c>
-      <c r="K30">
-        <v>0</v>
-      </c>
-      <c r="L30">
-        <v>0</v>
-      </c>
-      <c r="M30" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N30" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K30" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L30" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A31" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B31">
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D31" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E31">
         <v>10</v>
@@ -1953,31 +1858,25 @@
       <c r="J31">
         <v>82</v>
       </c>
-      <c r="K31">
-        <v>0</v>
-      </c>
-      <c r="L31">
-        <v>0</v>
-      </c>
-      <c r="M31" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N31" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K31" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L31" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A32" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B32">
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D32" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E32">
         <v>24</v>
@@ -1997,31 +1896,25 @@
       <c r="J32">
         <v>47</v>
       </c>
-      <c r="K32">
-        <v>0</v>
-      </c>
-      <c r="L32">
-        <v>0</v>
-      </c>
-      <c r="M32" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N32" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K32" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L32" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A33" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B33">
         <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D33" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E33">
         <v>18</v>
@@ -2041,31 +1934,25 @@
       <c r="J33">
         <v>66</v>
       </c>
-      <c r="K33">
-        <v>0</v>
-      </c>
-      <c r="L33">
-        <v>0</v>
-      </c>
-      <c r="M33" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N33" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K33" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L33" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A34" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B34">
         <v>1</v>
       </c>
       <c r="C34" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D34" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E34">
         <v>20</v>
@@ -2085,31 +1972,25 @@
       <c r="J34">
         <v>89</v>
       </c>
-      <c r="K34">
-        <v>0</v>
-      </c>
-      <c r="L34">
-        <v>0</v>
-      </c>
-      <c r="M34" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N34" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K34" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L34" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A35" t="s">
+        <v>22</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>46</v>
+      </c>
+      <c r="D35" t="s">
         <v>24</v>
-      </c>
-      <c r="B35">
-        <v>1</v>
-      </c>
-      <c r="C35" t="s">
-        <v>48</v>
-      </c>
-      <c r="D35" t="s">
-        <v>26</v>
       </c>
       <c r="E35">
         <v>14</v>
@@ -2129,31 +2010,25 @@
       <c r="J35">
         <v>76</v>
       </c>
-      <c r="K35">
-        <v>0</v>
-      </c>
-      <c r="L35">
-        <v>0</v>
-      </c>
-      <c r="M35" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N35" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K35" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L35" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A36" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B36">
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D36" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E36">
         <v>7</v>
@@ -2173,31 +2048,25 @@
       <c r="J36">
         <v>46</v>
       </c>
-      <c r="K36">
-        <v>0</v>
-      </c>
-      <c r="L36">
-        <v>0</v>
-      </c>
-      <c r="M36" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N36" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K36" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L36" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A37" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B37">
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D37" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E37">
         <v>27</v>
@@ -2217,31 +2086,25 @@
       <c r="J37">
         <v>100</v>
       </c>
-      <c r="K37">
-        <v>0</v>
-      </c>
-      <c r="L37">
-        <v>0</v>
-      </c>
-      <c r="M37" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N37" t="s">
+      <c r="K37" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L37" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A38" t="s">
+        <v>48</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>50</v>
-      </c>
-      <c r="B38">
-        <v>1</v>
-      </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
         <v>51</v>
-      </c>
-      <c r="D38" t="s">
-        <v>53</v>
       </c>
       <c r="E38">
         <v>283</v>
@@ -2261,17 +2124,1417 @@
       <c r="J38">
         <v>92</v>
       </c>
-      <c r="K38">
-        <v>0</v>
-      </c>
-      <c r="L38">
-        <v>0</v>
-      </c>
-      <c r="M38" s="2">
-        <v>45993</v>
-      </c>
-      <c r="N38" t="s">
+      <c r="K38" s="2">
+        <v>45993</v>
+      </c>
+      <c r="L38" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A39" t="s">
         <v>52</v>
+      </c>
+      <c r="B39">
+        <v>2</v>
+      </c>
+      <c r="C39" t="s">
+        <v>65</v>
+      </c>
+      <c r="D39" t="s">
+        <v>24</v>
+      </c>
+      <c r="E39">
+        <v>25</v>
+      </c>
+      <c r="F39">
+        <v>25</v>
+      </c>
+      <c r="G39">
+        <v>100</v>
+      </c>
+      <c r="H39">
+        <v>138</v>
+      </c>
+      <c r="I39">
+        <v>227</v>
+      </c>
+      <c r="J39">
+        <v>61</v>
+      </c>
+      <c r="K39" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L39" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A40" t="s">
+        <v>52</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>65</v>
+      </c>
+      <c r="D40" t="s">
+        <v>25</v>
+      </c>
+      <c r="E40">
+        <v>42</v>
+      </c>
+      <c r="F40">
+        <v>42</v>
+      </c>
+      <c r="G40">
+        <v>100</v>
+      </c>
+      <c r="H40">
+        <v>170</v>
+      </c>
+      <c r="I40">
+        <v>227</v>
+      </c>
+      <c r="J40">
+        <v>75</v>
+      </c>
+      <c r="K40" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L40" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A41" t="s">
+        <v>52</v>
+      </c>
+      <c r="B41">
+        <v>2</v>
+      </c>
+      <c r="C41" t="s">
+        <v>65</v>
+      </c>
+      <c r="D41" t="s">
+        <v>26</v>
+      </c>
+      <c r="E41">
+        <v>9</v>
+      </c>
+      <c r="F41">
+        <v>9</v>
+      </c>
+      <c r="G41">
+        <v>100</v>
+      </c>
+      <c r="H41">
+        <v>173</v>
+      </c>
+      <c r="I41">
+        <v>227</v>
+      </c>
+      <c r="J41">
+        <v>76</v>
+      </c>
+      <c r="K41" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L41" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A42" t="s">
+        <v>53</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>66</v>
+      </c>
+      <c r="D42" t="s">
+        <v>24</v>
+      </c>
+      <c r="E42">
+        <v>36</v>
+      </c>
+      <c r="F42">
+        <v>36</v>
+      </c>
+      <c r="G42">
+        <v>100</v>
+      </c>
+      <c r="H42">
+        <v>90</v>
+      </c>
+      <c r="I42">
+        <v>95</v>
+      </c>
+      <c r="J42">
+        <v>95</v>
+      </c>
+      <c r="K42" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L42" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A43" t="s">
+        <v>53</v>
+      </c>
+      <c r="B43">
+        <v>2</v>
+      </c>
+      <c r="C43" t="s">
+        <v>66</v>
+      </c>
+      <c r="D43" t="s">
+        <v>25</v>
+      </c>
+      <c r="E43">
+        <v>17</v>
+      </c>
+      <c r="F43">
+        <v>17</v>
+      </c>
+      <c r="G43">
+        <v>100</v>
+      </c>
+      <c r="H43">
+        <v>46</v>
+      </c>
+      <c r="I43">
+        <v>95</v>
+      </c>
+      <c r="J43">
+        <v>38</v>
+      </c>
+      <c r="K43" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L43" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A44" t="s">
+        <v>53</v>
+      </c>
+      <c r="B44">
+        <v>2</v>
+      </c>
+      <c r="C44" t="s">
+        <v>66</v>
+      </c>
+      <c r="D44" t="s">
+        <v>26</v>
+      </c>
+      <c r="E44">
+        <v>4</v>
+      </c>
+      <c r="F44">
+        <v>4</v>
+      </c>
+      <c r="G44">
+        <v>100</v>
+      </c>
+      <c r="H44">
+        <v>78</v>
+      </c>
+      <c r="I44">
+        <v>95</v>
+      </c>
+      <c r="J44">
+        <v>82</v>
+      </c>
+      <c r="K44" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L44" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A45" t="s">
+        <v>54</v>
+      </c>
+      <c r="B45">
+        <v>2</v>
+      </c>
+      <c r="C45" t="s">
+        <v>67</v>
+      </c>
+      <c r="D45" t="s">
+        <v>24</v>
+      </c>
+      <c r="E45">
+        <v>21</v>
+      </c>
+      <c r="F45">
+        <v>21</v>
+      </c>
+      <c r="G45">
+        <v>100</v>
+      </c>
+      <c r="H45">
+        <v>124</v>
+      </c>
+      <c r="I45">
+        <v>128</v>
+      </c>
+      <c r="J45">
+        <v>97</v>
+      </c>
+      <c r="K45" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L45" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A46" t="s">
+        <v>54</v>
+      </c>
+      <c r="B46">
+        <v>2</v>
+      </c>
+      <c r="C46" t="s">
+        <v>67</v>
+      </c>
+      <c r="D46" t="s">
+        <v>25</v>
+      </c>
+      <c r="E46">
+        <v>19</v>
+      </c>
+      <c r="F46">
+        <v>19</v>
+      </c>
+      <c r="G46">
+        <v>100</v>
+      </c>
+      <c r="H46">
+        <v>114</v>
+      </c>
+      <c r="I46">
+        <v>128</v>
+      </c>
+      <c r="J46">
+        <v>89</v>
+      </c>
+      <c r="K46" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L46" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A47" t="s">
+        <v>54</v>
+      </c>
+      <c r="B47">
+        <v>2</v>
+      </c>
+      <c r="C47" t="s">
+        <v>67</v>
+      </c>
+      <c r="D47" t="s">
+        <v>26</v>
+      </c>
+      <c r="E47">
+        <v>3</v>
+      </c>
+      <c r="F47">
+        <v>3</v>
+      </c>
+      <c r="G47">
+        <v>100</v>
+      </c>
+      <c r="H47">
+        <v>98</v>
+      </c>
+      <c r="I47">
+        <v>128</v>
+      </c>
+      <c r="J47">
+        <v>77</v>
+      </c>
+      <c r="K47" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L47" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A48" t="s">
+        <v>55</v>
+      </c>
+      <c r="B48">
+        <v>2</v>
+      </c>
+      <c r="C48" t="s">
+        <v>68</v>
+      </c>
+      <c r="D48" t="s">
+        <v>24</v>
+      </c>
+      <c r="E48">
+        <v>21</v>
+      </c>
+      <c r="F48">
+        <v>21</v>
+      </c>
+      <c r="G48">
+        <v>100</v>
+      </c>
+      <c r="H48">
+        <v>124</v>
+      </c>
+      <c r="I48">
+        <v>128</v>
+      </c>
+      <c r="J48">
+        <v>97</v>
+      </c>
+      <c r="K48" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L48" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A49" t="s">
+        <v>55</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49" t="s">
+        <v>68</v>
+      </c>
+      <c r="D49" t="s">
+        <v>25</v>
+      </c>
+      <c r="E49">
+        <v>19</v>
+      </c>
+      <c r="F49">
+        <v>19</v>
+      </c>
+      <c r="G49">
+        <v>100</v>
+      </c>
+      <c r="H49">
+        <v>114</v>
+      </c>
+      <c r="I49">
+        <v>128</v>
+      </c>
+      <c r="J49">
+        <v>89</v>
+      </c>
+      <c r="K49" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L49" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A50" t="s">
+        <v>55</v>
+      </c>
+      <c r="B50">
+        <v>2</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50" t="s">
+        <v>26</v>
+      </c>
+      <c r="E50">
+        <v>3</v>
+      </c>
+      <c r="F50">
+        <v>3</v>
+      </c>
+      <c r="G50">
+        <v>100</v>
+      </c>
+      <c r="H50">
+        <v>98</v>
+      </c>
+      <c r="I50">
+        <v>128</v>
+      </c>
+      <c r="J50">
+        <v>77</v>
+      </c>
+      <c r="K50" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L50" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A51" t="s">
+        <v>56</v>
+      </c>
+      <c r="B51">
+        <v>2</v>
+      </c>
+      <c r="C51" t="s">
+        <v>69</v>
+      </c>
+      <c r="D51" t="s">
+        <v>24</v>
+      </c>
+      <c r="E51">
+        <v>14</v>
+      </c>
+      <c r="F51">
+        <v>14</v>
+      </c>
+      <c r="G51">
+        <v>100</v>
+      </c>
+      <c r="H51">
+        <v>110</v>
+      </c>
+      <c r="I51">
+        <v>199</v>
+      </c>
+      <c r="J51">
+        <v>55</v>
+      </c>
+      <c r="K51" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L51" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A52" t="s">
+        <v>56</v>
+      </c>
+      <c r="B52">
+        <v>2</v>
+      </c>
+      <c r="C52" t="s">
+        <v>69</v>
+      </c>
+      <c r="D52" t="s">
+        <v>25</v>
+      </c>
+      <c r="E52">
+        <v>36</v>
+      </c>
+      <c r="F52">
+        <v>36</v>
+      </c>
+      <c r="G52">
+        <v>100</v>
+      </c>
+      <c r="H52">
+        <v>142</v>
+      </c>
+      <c r="I52">
+        <v>199</v>
+      </c>
+      <c r="J52">
+        <v>71</v>
+      </c>
+      <c r="K52" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L52" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A53" t="s">
+        <v>56</v>
+      </c>
+      <c r="B53">
+        <v>2</v>
+      </c>
+      <c r="C53" t="s">
+        <v>69</v>
+      </c>
+      <c r="D53" t="s">
+        <v>26</v>
+      </c>
+      <c r="E53">
+        <v>5</v>
+      </c>
+      <c r="F53">
+        <v>5</v>
+      </c>
+      <c r="G53">
+        <v>100</v>
+      </c>
+      <c r="H53">
+        <v>145</v>
+      </c>
+      <c r="I53">
+        <v>199</v>
+      </c>
+      <c r="J53">
+        <v>73</v>
+      </c>
+      <c r="K53" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L53" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A54" t="s">
+        <v>57</v>
+      </c>
+      <c r="B54">
+        <v>2</v>
+      </c>
+      <c r="C54" t="s">
+        <v>70</v>
+      </c>
+      <c r="D54" t="s">
+        <v>24</v>
+      </c>
+      <c r="E54">
+        <v>14</v>
+      </c>
+      <c r="F54">
+        <v>14</v>
+      </c>
+      <c r="G54">
+        <v>100</v>
+      </c>
+      <c r="H54">
+        <v>110</v>
+      </c>
+      <c r="I54">
+        <v>199</v>
+      </c>
+      <c r="J54">
+        <v>55</v>
+      </c>
+      <c r="K54" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L54" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A55" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55">
+        <v>2</v>
+      </c>
+      <c r="C55" t="s">
+        <v>70</v>
+      </c>
+      <c r="D55" t="s">
+        <v>25</v>
+      </c>
+      <c r="E55">
+        <v>36</v>
+      </c>
+      <c r="F55">
+        <v>36</v>
+      </c>
+      <c r="G55">
+        <v>100</v>
+      </c>
+      <c r="H55">
+        <v>142</v>
+      </c>
+      <c r="I55">
+        <v>199</v>
+      </c>
+      <c r="J55">
+        <v>71</v>
+      </c>
+      <c r="K55" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L55" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A56" t="s">
+        <v>57</v>
+      </c>
+      <c r="B56">
+        <v>2</v>
+      </c>
+      <c r="C56" t="s">
+        <v>70</v>
+      </c>
+      <c r="D56" t="s">
+        <v>26</v>
+      </c>
+      <c r="E56">
+        <v>5</v>
+      </c>
+      <c r="F56">
+        <v>5</v>
+      </c>
+      <c r="G56">
+        <v>100</v>
+      </c>
+      <c r="H56">
+        <v>145</v>
+      </c>
+      <c r="I56">
+        <v>199</v>
+      </c>
+      <c r="J56">
+        <v>73</v>
+      </c>
+      <c r="K56" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L56" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A57" t="s">
+        <v>58</v>
+      </c>
+      <c r="B57">
+        <v>2</v>
+      </c>
+      <c r="C57" t="s">
+        <v>71</v>
+      </c>
+      <c r="D57" t="s">
+        <v>24</v>
+      </c>
+      <c r="E57">
+        <v>36</v>
+      </c>
+      <c r="F57">
+        <v>36</v>
+      </c>
+      <c r="G57">
+        <v>100</v>
+      </c>
+      <c r="H57">
+        <v>90</v>
+      </c>
+      <c r="I57">
+        <v>95</v>
+      </c>
+      <c r="J57">
+        <v>95</v>
+      </c>
+      <c r="K57" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L57" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A58" t="s">
+        <v>58</v>
+      </c>
+      <c r="B58">
+        <v>2</v>
+      </c>
+      <c r="C58" t="s">
+        <v>71</v>
+      </c>
+      <c r="D58" t="s">
+        <v>25</v>
+      </c>
+      <c r="E58">
+        <v>17</v>
+      </c>
+      <c r="F58">
+        <v>17</v>
+      </c>
+      <c r="G58">
+        <v>100</v>
+      </c>
+      <c r="H58">
+        <v>46</v>
+      </c>
+      <c r="I58">
+        <v>95</v>
+      </c>
+      <c r="J58">
+        <v>38</v>
+      </c>
+      <c r="K58" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L58" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A59" t="s">
+        <v>58</v>
+      </c>
+      <c r="B59">
+        <v>2</v>
+      </c>
+      <c r="C59" t="s">
+        <v>71</v>
+      </c>
+      <c r="D59" t="s">
+        <v>26</v>
+      </c>
+      <c r="E59">
+        <v>4</v>
+      </c>
+      <c r="F59">
+        <v>4</v>
+      </c>
+      <c r="G59">
+        <v>100</v>
+      </c>
+      <c r="H59">
+        <v>78</v>
+      </c>
+      <c r="I59">
+        <v>95</v>
+      </c>
+      <c r="J59">
+        <v>82</v>
+      </c>
+      <c r="K59" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L59" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A60" t="s">
+        <v>59</v>
+      </c>
+      <c r="B60">
+        <v>2</v>
+      </c>
+      <c r="C60" t="s">
+        <v>72</v>
+      </c>
+      <c r="D60" t="s">
+        <v>24</v>
+      </c>
+      <c r="E60">
+        <v>36</v>
+      </c>
+      <c r="F60">
+        <v>36</v>
+      </c>
+      <c r="G60">
+        <v>100</v>
+      </c>
+      <c r="H60">
+        <v>90</v>
+      </c>
+      <c r="I60">
+        <v>95</v>
+      </c>
+      <c r="J60">
+        <v>95</v>
+      </c>
+      <c r="K60" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L60" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A61" t="s">
+        <v>59</v>
+      </c>
+      <c r="B61">
+        <v>2</v>
+      </c>
+      <c r="C61" t="s">
+        <v>72</v>
+      </c>
+      <c r="D61" t="s">
+        <v>25</v>
+      </c>
+      <c r="E61">
+        <v>17</v>
+      </c>
+      <c r="F61">
+        <v>17</v>
+      </c>
+      <c r="G61">
+        <v>100</v>
+      </c>
+      <c r="H61">
+        <v>46</v>
+      </c>
+      <c r="I61">
+        <v>95</v>
+      </c>
+      <c r="J61">
+        <v>38</v>
+      </c>
+      <c r="K61" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L61" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A62" t="s">
+        <v>59</v>
+      </c>
+      <c r="B62">
+        <v>2</v>
+      </c>
+      <c r="C62" t="s">
+        <v>72</v>
+      </c>
+      <c r="D62" t="s">
+        <v>26</v>
+      </c>
+      <c r="E62">
+        <v>4</v>
+      </c>
+      <c r="F62">
+        <v>4</v>
+      </c>
+      <c r="G62">
+        <v>100</v>
+      </c>
+      <c r="H62">
+        <v>78</v>
+      </c>
+      <c r="I62">
+        <v>95</v>
+      </c>
+      <c r="J62">
+        <v>82</v>
+      </c>
+      <c r="K62" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L62" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A63" t="s">
+        <v>60</v>
+      </c>
+      <c r="B63">
+        <v>2</v>
+      </c>
+      <c r="C63" t="s">
+        <v>73</v>
+      </c>
+      <c r="D63" t="s">
+        <v>24</v>
+      </c>
+      <c r="E63">
+        <v>21</v>
+      </c>
+      <c r="F63">
+        <v>21</v>
+      </c>
+      <c r="G63">
+        <v>100</v>
+      </c>
+      <c r="H63">
+        <v>124</v>
+      </c>
+      <c r="I63">
+        <v>128</v>
+      </c>
+      <c r="J63">
+        <v>97</v>
+      </c>
+      <c r="K63" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L63" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A64" t="s">
+        <v>60</v>
+      </c>
+      <c r="B64">
+        <v>2</v>
+      </c>
+      <c r="C64" t="s">
+        <v>73</v>
+      </c>
+      <c r="D64" t="s">
+        <v>25</v>
+      </c>
+      <c r="E64">
+        <v>19</v>
+      </c>
+      <c r="F64">
+        <v>19</v>
+      </c>
+      <c r="G64">
+        <v>100</v>
+      </c>
+      <c r="H64">
+        <v>114</v>
+      </c>
+      <c r="I64">
+        <v>128</v>
+      </c>
+      <c r="J64">
+        <v>89</v>
+      </c>
+      <c r="K64" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L64" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A65" t="s">
+        <v>60</v>
+      </c>
+      <c r="B65">
+        <v>2</v>
+      </c>
+      <c r="C65" t="s">
+        <v>73</v>
+      </c>
+      <c r="D65" t="s">
+        <v>26</v>
+      </c>
+      <c r="E65">
+        <v>3</v>
+      </c>
+      <c r="F65">
+        <v>3</v>
+      </c>
+      <c r="G65">
+        <v>100</v>
+      </c>
+      <c r="H65">
+        <v>98</v>
+      </c>
+      <c r="I65">
+        <v>128</v>
+      </c>
+      <c r="J65">
+        <v>77</v>
+      </c>
+      <c r="K65" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L65" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A66" t="s">
+        <v>61</v>
+      </c>
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66" t="s">
+        <v>74</v>
+      </c>
+      <c r="D66" t="s">
+        <v>24</v>
+      </c>
+      <c r="E66">
+        <v>14</v>
+      </c>
+      <c r="F66">
+        <v>14</v>
+      </c>
+      <c r="G66">
+        <v>100</v>
+      </c>
+      <c r="H66">
+        <v>110</v>
+      </c>
+      <c r="I66">
+        <v>199</v>
+      </c>
+      <c r="J66">
+        <v>55</v>
+      </c>
+      <c r="K66" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L66" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A67" t="s">
+        <v>61</v>
+      </c>
+      <c r="B67">
+        <v>2</v>
+      </c>
+      <c r="C67" t="s">
+        <v>74</v>
+      </c>
+      <c r="D67" t="s">
+        <v>25</v>
+      </c>
+      <c r="E67">
+        <v>36</v>
+      </c>
+      <c r="F67">
+        <v>36</v>
+      </c>
+      <c r="G67">
+        <v>100</v>
+      </c>
+      <c r="H67">
+        <v>142</v>
+      </c>
+      <c r="I67">
+        <v>199</v>
+      </c>
+      <c r="J67">
+        <v>71</v>
+      </c>
+      <c r="K67" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L67" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A68" t="s">
+        <v>61</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>74</v>
+      </c>
+      <c r="D68" t="s">
+        <v>26</v>
+      </c>
+      <c r="E68">
+        <v>5</v>
+      </c>
+      <c r="F68">
+        <v>5</v>
+      </c>
+      <c r="G68">
+        <v>100</v>
+      </c>
+      <c r="H68">
+        <v>145</v>
+      </c>
+      <c r="I68">
+        <v>199</v>
+      </c>
+      <c r="J68">
+        <v>73</v>
+      </c>
+      <c r="K68" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L68" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A69" t="s">
+        <v>62</v>
+      </c>
+      <c r="B69">
+        <v>2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>75</v>
+      </c>
+      <c r="D69" t="s">
+        <v>24</v>
+      </c>
+      <c r="E69">
+        <v>19</v>
+      </c>
+      <c r="F69">
+        <v>19</v>
+      </c>
+      <c r="G69">
+        <v>100</v>
+      </c>
+      <c r="H69">
+        <v>75</v>
+      </c>
+      <c r="I69">
+        <v>96</v>
+      </c>
+      <c r="J69">
+        <v>78</v>
+      </c>
+      <c r="K69" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L69" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A70" t="s">
+        <v>62</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>75</v>
+      </c>
+      <c r="D70" t="s">
+        <v>25</v>
+      </c>
+      <c r="E70">
+        <v>11</v>
+      </c>
+      <c r="F70">
+        <v>11</v>
+      </c>
+      <c r="G70">
+        <v>100</v>
+      </c>
+      <c r="H70">
+        <v>38</v>
+      </c>
+      <c r="I70">
+        <v>96</v>
+      </c>
+      <c r="J70">
+        <v>40</v>
+      </c>
+      <c r="K70" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L70" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A71" t="s">
+        <v>62</v>
+      </c>
+      <c r="B71">
+        <v>2</v>
+      </c>
+      <c r="C71" t="s">
+        <v>75</v>
+      </c>
+      <c r="D71" t="s">
+        <v>26</v>
+      </c>
+      <c r="E71">
+        <v>4</v>
+      </c>
+      <c r="F71">
+        <v>4</v>
+      </c>
+      <c r="G71">
+        <v>100</v>
+      </c>
+      <c r="H71">
+        <v>61</v>
+      </c>
+      <c r="I71">
+        <v>96</v>
+      </c>
+      <c r="J71">
+        <v>64</v>
+      </c>
+      <c r="K71" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L71" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A72" t="s">
+        <v>63</v>
+      </c>
+      <c r="B72">
+        <v>2</v>
+      </c>
+      <c r="C72" t="s">
+        <v>76</v>
+      </c>
+      <c r="D72" t="s">
+        <v>24</v>
+      </c>
+      <c r="E72">
+        <v>19</v>
+      </c>
+      <c r="F72">
+        <v>19</v>
+      </c>
+      <c r="G72">
+        <v>100</v>
+      </c>
+      <c r="H72">
+        <v>75</v>
+      </c>
+      <c r="I72">
+        <v>96</v>
+      </c>
+      <c r="J72">
+        <v>78</v>
+      </c>
+      <c r="K72" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L72" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A73" t="s">
+        <v>63</v>
+      </c>
+      <c r="B73">
+        <v>2</v>
+      </c>
+      <c r="C73" t="s">
+        <v>76</v>
+      </c>
+      <c r="D73" t="s">
+        <v>25</v>
+      </c>
+      <c r="E73">
+        <v>11</v>
+      </c>
+      <c r="F73">
+        <v>11</v>
+      </c>
+      <c r="G73">
+        <v>100</v>
+      </c>
+      <c r="H73">
+        <v>38</v>
+      </c>
+      <c r="I73">
+        <v>96</v>
+      </c>
+      <c r="J73">
+        <v>40</v>
+      </c>
+      <c r="K73" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L73" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A74" t="s">
+        <v>63</v>
+      </c>
+      <c r="B74">
+        <v>2</v>
+      </c>
+      <c r="C74" t="s">
+        <v>76</v>
+      </c>
+      <c r="D74" t="s">
+        <v>26</v>
+      </c>
+      <c r="E74">
+        <v>4</v>
+      </c>
+      <c r="F74">
+        <v>4</v>
+      </c>
+      <c r="G74">
+        <v>100</v>
+      </c>
+      <c r="H74">
+        <v>61</v>
+      </c>
+      <c r="I74">
+        <v>96</v>
+      </c>
+      <c r="J74">
+        <v>64</v>
+      </c>
+      <c r="K74" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L74" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A75" t="s">
+        <v>48</v>
+      </c>
+      <c r="B75">
+        <v>2</v>
+      </c>
+      <c r="C75" t="s">
+        <v>64</v>
+      </c>
+      <c r="D75" t="s">
+        <v>51</v>
+      </c>
+      <c r="E75">
+        <v>510</v>
+      </c>
+      <c r="F75">
+        <v>510</v>
+      </c>
+      <c r="G75">
+        <v>100</v>
+      </c>
+      <c r="H75">
+        <v>505</v>
+      </c>
+      <c r="I75">
+        <v>546</v>
+      </c>
+      <c r="J75">
+        <v>92</v>
+      </c>
+      <c r="K75" s="2">
+        <v>46009</v>
+      </c>
+      <c r="L75" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sprint 3 coverage_report.xlsx updated info
</commit_message>
<xml_diff>
--- a/Evidence/MA/coverage_report.xlsx
+++ b/Evidence/MA/coverage_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raygu\Downloads\CO3095\Evidence\MA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B83393EE-DEBA-4895-9F07-DD0B2AB4E5E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4471854-6991-423E-9D05-24281E973204}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="16186" xr2:uid="{B4F26AE1-5879-47D9-8144-9A3C1A46093E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="113">
   <si>
     <t>Story ID</t>
   </si>
@@ -285,6 +285,96 @@
   </si>
   <si>
     <t>playlist_model, playlists_basic, playlists_edit, playlists_advanced, library_search_scan</t>
+  </si>
+  <si>
+    <t>S3-01</t>
+  </si>
+  <si>
+    <t>S3-02</t>
+  </si>
+  <si>
+    <t>S3-03</t>
+  </si>
+  <si>
+    <t>S3-04</t>
+  </si>
+  <si>
+    <t>S3-05</t>
+  </si>
+  <si>
+    <t>S3-06</t>
+  </si>
+  <si>
+    <t>S3-07</t>
+  </si>
+  <si>
+    <t>S3-08</t>
+  </si>
+  <si>
+    <t>S3-09</t>
+  </si>
+  <si>
+    <t>S3-10</t>
+  </si>
+  <si>
+    <t>S3-11</t>
+  </si>
+  <si>
+    <t>S3-12</t>
+  </si>
+  <si>
+    <t>Sprint 3 Total Coverage</t>
+  </si>
+  <si>
+    <t>Shuffle</t>
+  </si>
+  <si>
+    <t>Loop</t>
+  </si>
+  <si>
+    <t>Show Queue</t>
+  </si>
+  <si>
+    <t>add/remove songs in queue</t>
+  </si>
+  <si>
+    <t>play next</t>
+  </si>
+  <si>
+    <t>clear queue</t>
+  </si>
+  <si>
+    <t>playback speed</t>
+  </si>
+  <si>
+    <t>like songs</t>
+  </si>
+  <si>
+    <t>view liked songs</t>
+  </si>
+  <si>
+    <t>sort playlist</t>
+  </si>
+  <si>
+    <t>top songs</t>
+  </si>
+  <si>
+    <t>sleep timer</t>
+  </si>
+  <si>
+    <t>player_core, player_queue, playlists_basic, player_metrics</t>
+  </si>
+  <si>
+    <t>player_metrics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">player_core, player_queue </t>
+  </si>
+  <si>
+    <t>Sprint 4 Total Coverate</t>
+  </si>
+  <si>
+    <t>All Code Modules</t>
   </si>
 </sst>
 </file>
@@ -672,7 +762,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6C833DE-F332-4BAA-A701-CCE6281E1DB6}">
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:L140"/>
   <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="3" max="3" width="29.52734375" customWidth="1"/>
@@ -3537,6 +3627,1483 @@
         <v>82</v>
       </c>
     </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A76" t="s">
+        <v>83</v>
+      </c>
+      <c r="B76">
+        <v>3</v>
+      </c>
+      <c r="C76" t="s">
+        <v>96</v>
+      </c>
+      <c r="D76" t="s">
+        <v>25</v>
+      </c>
+      <c r="E76">
+        <v>54</v>
+      </c>
+      <c r="F76">
+        <v>54</v>
+      </c>
+      <c r="G76">
+        <v>100</v>
+      </c>
+      <c r="H76">
+        <v>296</v>
+      </c>
+      <c r="I76">
+        <v>533</v>
+      </c>
+      <c r="J76">
+        <v>56</v>
+      </c>
+      <c r="K76" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L76" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A77" t="s">
+        <v>83</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77" t="s">
+        <v>96</v>
+      </c>
+      <c r="D77" t="s">
+        <v>26</v>
+      </c>
+      <c r="E77">
+        <v>14</v>
+      </c>
+      <c r="F77">
+        <v>14</v>
+      </c>
+      <c r="G77">
+        <v>100</v>
+      </c>
+      <c r="H77">
+        <v>316</v>
+      </c>
+      <c r="I77">
+        <v>533</v>
+      </c>
+      <c r="J77">
+        <v>59</v>
+      </c>
+      <c r="K77" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L77" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A78" t="s">
+        <v>84</v>
+      </c>
+      <c r="B78">
+        <v>3</v>
+      </c>
+      <c r="C78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D78" t="s">
+        <v>25</v>
+      </c>
+      <c r="E78">
+        <v>54</v>
+      </c>
+      <c r="F78">
+        <v>54</v>
+      </c>
+      <c r="G78">
+        <v>100</v>
+      </c>
+      <c r="H78">
+        <v>296</v>
+      </c>
+      <c r="I78">
+        <v>533</v>
+      </c>
+      <c r="J78">
+        <v>56</v>
+      </c>
+      <c r="K78" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L78" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A79" t="s">
+        <v>84</v>
+      </c>
+      <c r="B79">
+        <v>3</v>
+      </c>
+      <c r="C79" t="s">
+        <v>97</v>
+      </c>
+      <c r="D79" t="s">
+        <v>26</v>
+      </c>
+      <c r="E79">
+        <v>14</v>
+      </c>
+      <c r="F79">
+        <v>14</v>
+      </c>
+      <c r="G79">
+        <v>100</v>
+      </c>
+      <c r="H79">
+        <v>316</v>
+      </c>
+      <c r="I79">
+        <v>533</v>
+      </c>
+      <c r="J79">
+        <v>59</v>
+      </c>
+      <c r="K79" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L79" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A80" t="s">
+        <v>85</v>
+      </c>
+      <c r="B80">
+        <v>3</v>
+      </c>
+      <c r="C80" t="s">
+        <v>98</v>
+      </c>
+      <c r="D80" t="s">
+        <v>25</v>
+      </c>
+      <c r="E80">
+        <v>54</v>
+      </c>
+      <c r="F80">
+        <v>54</v>
+      </c>
+      <c r="G80">
+        <v>100</v>
+      </c>
+      <c r="H80">
+        <v>296</v>
+      </c>
+      <c r="I80">
+        <v>533</v>
+      </c>
+      <c r="J80">
+        <v>56</v>
+      </c>
+      <c r="K80" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L80" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A81" t="s">
+        <v>85</v>
+      </c>
+      <c r="B81">
+        <v>3</v>
+      </c>
+      <c r="C81" t="s">
+        <v>98</v>
+      </c>
+      <c r="D81" t="s">
+        <v>26</v>
+      </c>
+      <c r="E81">
+        <v>14</v>
+      </c>
+      <c r="F81">
+        <v>14</v>
+      </c>
+      <c r="G81">
+        <v>100</v>
+      </c>
+      <c r="H81">
+        <v>316</v>
+      </c>
+      <c r="I81">
+        <v>533</v>
+      </c>
+      <c r="J81">
+        <v>59</v>
+      </c>
+      <c r="K81" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L81" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A82" t="s">
+        <v>86</v>
+      </c>
+      <c r="B82">
+        <v>3</v>
+      </c>
+      <c r="C82" t="s">
+        <v>99</v>
+      </c>
+      <c r="D82" t="s">
+        <v>25</v>
+      </c>
+      <c r="E82">
+        <v>54</v>
+      </c>
+      <c r="F82">
+        <v>54</v>
+      </c>
+      <c r="G82">
+        <v>100</v>
+      </c>
+      <c r="H82">
+        <v>296</v>
+      </c>
+      <c r="I82">
+        <v>533</v>
+      </c>
+      <c r="J82">
+        <v>56</v>
+      </c>
+      <c r="K82" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L82" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A83" t="s">
+        <v>86</v>
+      </c>
+      <c r="B83">
+        <v>3</v>
+      </c>
+      <c r="C83" t="s">
+        <v>99</v>
+      </c>
+      <c r="D83" t="s">
+        <v>26</v>
+      </c>
+      <c r="E83">
+        <v>14</v>
+      </c>
+      <c r="F83">
+        <v>14</v>
+      </c>
+      <c r="G83">
+        <v>100</v>
+      </c>
+      <c r="H83">
+        <v>316</v>
+      </c>
+      <c r="I83">
+        <v>533</v>
+      </c>
+      <c r="J83">
+        <v>59</v>
+      </c>
+      <c r="K83" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L83" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A84" t="s">
+        <v>87</v>
+      </c>
+      <c r="B84">
+        <v>3</v>
+      </c>
+      <c r="C84" t="s">
+        <v>100</v>
+      </c>
+      <c r="D84" t="s">
+        <v>25</v>
+      </c>
+      <c r="E84">
+        <v>54</v>
+      </c>
+      <c r="F84">
+        <v>54</v>
+      </c>
+      <c r="G84">
+        <v>100</v>
+      </c>
+      <c r="H84">
+        <v>296</v>
+      </c>
+      <c r="I84">
+        <v>533</v>
+      </c>
+      <c r="J84">
+        <v>56</v>
+      </c>
+      <c r="K84" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L84" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A85" t="s">
+        <v>87</v>
+      </c>
+      <c r="B85">
+        <v>3</v>
+      </c>
+      <c r="C85" t="s">
+        <v>100</v>
+      </c>
+      <c r="D85" t="s">
+        <v>26</v>
+      </c>
+      <c r="E85">
+        <v>14</v>
+      </c>
+      <c r="F85">
+        <v>14</v>
+      </c>
+      <c r="G85">
+        <v>100</v>
+      </c>
+      <c r="H85">
+        <v>316</v>
+      </c>
+      <c r="I85">
+        <v>533</v>
+      </c>
+      <c r="J85">
+        <v>59</v>
+      </c>
+      <c r="K85" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L85" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A86" t="s">
+        <v>88</v>
+      </c>
+      <c r="B86">
+        <v>3</v>
+      </c>
+      <c r="C86" t="s">
+        <v>101</v>
+      </c>
+      <c r="D86" t="s">
+        <v>25</v>
+      </c>
+      <c r="E86">
+        <v>54</v>
+      </c>
+      <c r="F86">
+        <v>54</v>
+      </c>
+      <c r="G86">
+        <v>100</v>
+      </c>
+      <c r="H86">
+        <v>296</v>
+      </c>
+      <c r="I86">
+        <v>533</v>
+      </c>
+      <c r="J86">
+        <v>56</v>
+      </c>
+      <c r="K86" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L86" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A87" t="s">
+        <v>88</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="C87" t="s">
+        <v>101</v>
+      </c>
+      <c r="D87" t="s">
+        <v>26</v>
+      </c>
+      <c r="E87">
+        <v>14</v>
+      </c>
+      <c r="F87">
+        <v>14</v>
+      </c>
+      <c r="G87">
+        <v>100</v>
+      </c>
+      <c r="H87">
+        <v>316</v>
+      </c>
+      <c r="I87">
+        <v>533</v>
+      </c>
+      <c r="J87">
+        <v>59</v>
+      </c>
+      <c r="K87" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L87" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A88" t="s">
+        <v>89</v>
+      </c>
+      <c r="B88">
+        <v>3</v>
+      </c>
+      <c r="C88" t="s">
+        <v>102</v>
+      </c>
+      <c r="D88" t="s">
+        <v>24</v>
+      </c>
+      <c r="E88">
+        <v>11</v>
+      </c>
+      <c r="F88">
+        <v>11</v>
+      </c>
+      <c r="G88">
+        <v>100</v>
+      </c>
+      <c r="H88">
+        <v>87</v>
+      </c>
+      <c r="I88">
+        <v>678</v>
+      </c>
+      <c r="J88">
+        <v>13</v>
+      </c>
+      <c r="K88" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L88" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A89" t="s">
+        <v>89</v>
+      </c>
+      <c r="B89">
+        <v>3</v>
+      </c>
+      <c r="C89" t="s">
+        <v>102</v>
+      </c>
+      <c r="D89" t="s">
+        <v>25</v>
+      </c>
+      <c r="E89">
+        <v>83</v>
+      </c>
+      <c r="F89">
+        <v>83</v>
+      </c>
+      <c r="G89">
+        <v>100</v>
+      </c>
+      <c r="H89">
+        <v>377</v>
+      </c>
+      <c r="I89">
+        <v>678</v>
+      </c>
+      <c r="J89">
+        <v>56</v>
+      </c>
+      <c r="K89" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L89" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A90" t="s">
+        <v>89</v>
+      </c>
+      <c r="B90">
+        <v>3</v>
+      </c>
+      <c r="C90" t="s">
+        <v>102</v>
+      </c>
+      <c r="D90" t="s">
+        <v>26</v>
+      </c>
+      <c r="E90">
+        <v>23</v>
+      </c>
+      <c r="F90">
+        <v>23</v>
+      </c>
+      <c r="G90">
+        <v>100</v>
+      </c>
+      <c r="H90">
+        <v>414</v>
+      </c>
+      <c r="I90">
+        <v>678</v>
+      </c>
+      <c r="J90">
+        <v>61</v>
+      </c>
+      <c r="K90" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L90" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A91" t="s">
+        <v>90</v>
+      </c>
+      <c r="B91">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>103</v>
+      </c>
+      <c r="D91" t="s">
+        <v>24</v>
+      </c>
+      <c r="E91">
+        <v>26</v>
+      </c>
+      <c r="F91">
+        <v>26</v>
+      </c>
+      <c r="G91">
+        <v>100</v>
+      </c>
+      <c r="H91">
+        <v>104</v>
+      </c>
+      <c r="I91">
+        <v>141</v>
+      </c>
+      <c r="J91">
+        <v>74</v>
+      </c>
+      <c r="K91" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L91" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A92" t="s">
+        <v>90</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="s">
+        <v>103</v>
+      </c>
+      <c r="D92" t="s">
+        <v>25</v>
+      </c>
+      <c r="E92">
+        <v>14</v>
+      </c>
+      <c r="F92">
+        <v>14</v>
+      </c>
+      <c r="G92">
+        <v>100</v>
+      </c>
+      <c r="H92">
+        <v>46</v>
+      </c>
+      <c r="I92">
+        <v>141</v>
+      </c>
+      <c r="J92">
+        <v>33</v>
+      </c>
+      <c r="K92" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L92" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A93" t="s">
+        <v>91</v>
+      </c>
+      <c r="B93">
+        <v>3</v>
+      </c>
+      <c r="C93" t="s">
+        <v>104</v>
+      </c>
+      <c r="D93" t="s">
+        <v>24</v>
+      </c>
+      <c r="E93">
+        <v>26</v>
+      </c>
+      <c r="F93">
+        <v>26</v>
+      </c>
+      <c r="G93">
+        <v>100</v>
+      </c>
+      <c r="H93">
+        <v>104</v>
+      </c>
+      <c r="I93">
+        <v>141</v>
+      </c>
+      <c r="J93">
+        <v>74</v>
+      </c>
+      <c r="K93" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L93" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A94" t="s">
+        <v>91</v>
+      </c>
+      <c r="B94">
+        <v>3</v>
+      </c>
+      <c r="C94" t="s">
+        <v>104</v>
+      </c>
+      <c r="D94" t="s">
+        <v>25</v>
+      </c>
+      <c r="E94">
+        <v>14</v>
+      </c>
+      <c r="F94">
+        <v>14</v>
+      </c>
+      <c r="G94">
+        <v>100</v>
+      </c>
+      <c r="H94">
+        <v>46</v>
+      </c>
+      <c r="I94">
+        <v>141</v>
+      </c>
+      <c r="J94">
+        <v>33</v>
+      </c>
+      <c r="K94" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L94" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A95" t="s">
+        <v>92</v>
+      </c>
+      <c r="B95">
+        <v>3</v>
+      </c>
+      <c r="C95" t="s">
+        <v>105</v>
+      </c>
+      <c r="D95" t="s">
+        <v>24</v>
+      </c>
+      <c r="E95">
+        <v>7</v>
+      </c>
+      <c r="F95">
+        <v>7</v>
+      </c>
+      <c r="G95">
+        <v>100</v>
+      </c>
+      <c r="H95">
+        <v>115</v>
+      </c>
+      <c r="I95">
+        <v>255</v>
+      </c>
+      <c r="J95">
+        <v>45</v>
+      </c>
+      <c r="K95" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L95" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A96" t="s">
+        <v>92</v>
+      </c>
+      <c r="B96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>105</v>
+      </c>
+      <c r="D96" t="s">
+        <v>25</v>
+      </c>
+      <c r="E96">
+        <v>36</v>
+      </c>
+      <c r="F96">
+        <v>36</v>
+      </c>
+      <c r="G96">
+        <v>100</v>
+      </c>
+      <c r="H96">
+        <v>157</v>
+      </c>
+      <c r="I96">
+        <v>255</v>
+      </c>
+      <c r="J96">
+        <v>62</v>
+      </c>
+      <c r="K96" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L96" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="97" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A97" t="s">
+        <v>92</v>
+      </c>
+      <c r="B97">
+        <v>3</v>
+      </c>
+      <c r="C97" t="s">
+        <v>105</v>
+      </c>
+      <c r="D97" t="s">
+        <v>26</v>
+      </c>
+      <c r="E97">
+        <v>9</v>
+      </c>
+      <c r="F97">
+        <v>9</v>
+      </c>
+      <c r="G97">
+        <v>100</v>
+      </c>
+      <c r="H97">
+        <v>208</v>
+      </c>
+      <c r="I97">
+        <v>255</v>
+      </c>
+      <c r="J97">
+        <v>82</v>
+      </c>
+      <c r="K97" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L97" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="98" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A98" t="s">
+        <v>93</v>
+      </c>
+      <c r="B98">
+        <v>3</v>
+      </c>
+      <c r="C98" t="s">
+        <v>106</v>
+      </c>
+      <c r="D98" t="s">
+        <v>24</v>
+      </c>
+      <c r="E98">
+        <v>26</v>
+      </c>
+      <c r="F98">
+        <v>26</v>
+      </c>
+      <c r="G98">
+        <v>100</v>
+      </c>
+      <c r="H98">
+        <v>104</v>
+      </c>
+      <c r="I98">
+        <v>141</v>
+      </c>
+      <c r="J98">
+        <v>74</v>
+      </c>
+      <c r="K98" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L98" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="99" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A99" t="s">
+        <v>93</v>
+      </c>
+      <c r="B99">
+        <v>3</v>
+      </c>
+      <c r="C99" t="s">
+        <v>106</v>
+      </c>
+      <c r="D99" t="s">
+        <v>25</v>
+      </c>
+      <c r="E99">
+        <v>14</v>
+      </c>
+      <c r="F99">
+        <v>14</v>
+      </c>
+      <c r="G99">
+        <v>100</v>
+      </c>
+      <c r="H99">
+        <v>46</v>
+      </c>
+      <c r="I99">
+        <v>141</v>
+      </c>
+      <c r="J99">
+        <v>33</v>
+      </c>
+      <c r="K99" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L99" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="100" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A100" t="s">
+        <v>94</v>
+      </c>
+      <c r="B100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>107</v>
+      </c>
+      <c r="D100" t="s">
+        <v>24</v>
+      </c>
+      <c r="E100">
+        <v>11</v>
+      </c>
+      <c r="F100">
+        <v>11</v>
+      </c>
+      <c r="G100">
+        <v>100</v>
+      </c>
+      <c r="H100">
+        <v>72</v>
+      </c>
+      <c r="I100">
+        <v>145</v>
+      </c>
+      <c r="J100">
+        <v>50</v>
+      </c>
+      <c r="K100" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L100" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="101" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A101" t="s">
+        <v>94</v>
+      </c>
+      <c r="B101">
+        <v>3</v>
+      </c>
+      <c r="C101" t="s">
+        <v>107</v>
+      </c>
+      <c r="D101" t="s">
+        <v>25</v>
+      </c>
+      <c r="E101">
+        <v>29</v>
+      </c>
+      <c r="F101">
+        <v>29</v>
+      </c>
+      <c r="G101">
+        <v>100</v>
+      </c>
+      <c r="H101">
+        <v>81</v>
+      </c>
+      <c r="I101">
+        <v>145</v>
+      </c>
+      <c r="J101">
+        <v>56</v>
+      </c>
+      <c r="K101" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L101" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="102" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A102" t="s">
+        <v>94</v>
+      </c>
+      <c r="B102">
+        <v>3</v>
+      </c>
+      <c r="C102" t="s">
+        <v>107</v>
+      </c>
+      <c r="D102" t="s">
+        <v>26</v>
+      </c>
+      <c r="E102">
+        <v>9</v>
+      </c>
+      <c r="F102">
+        <v>9</v>
+      </c>
+      <c r="G102">
+        <v>100</v>
+      </c>
+      <c r="H102">
+        <v>98</v>
+      </c>
+      <c r="I102">
+        <v>145</v>
+      </c>
+      <c r="J102">
+        <v>68</v>
+      </c>
+      <c r="K102" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L102" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="103" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A103" t="s">
+        <v>48</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="s">
+        <v>95</v>
+      </c>
+      <c r="D103" t="s">
+        <v>51</v>
+      </c>
+      <c r="E103">
+        <v>209</v>
+      </c>
+      <c r="F103">
+        <v>209</v>
+      </c>
+      <c r="G103">
+        <v>100</v>
+      </c>
+      <c r="H103">
+        <v>853</v>
+      </c>
+      <c r="I103">
+        <v>1074</v>
+      </c>
+      <c r="J103">
+        <v>79</v>
+      </c>
+      <c r="K103" s="2">
+        <v>46024</v>
+      </c>
+      <c r="L103" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="104" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A104" t="s">
+        <v>52</v>
+      </c>
+      <c r="D104" t="s">
+        <v>24</v>
+      </c>
+      <c r="G104">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="105" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A105" t="s">
+        <v>52</v>
+      </c>
+      <c r="D105" t="s">
+        <v>25</v>
+      </c>
+      <c r="G105">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="106" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A106" t="s">
+        <v>52</v>
+      </c>
+      <c r="D106" t="s">
+        <v>26</v>
+      </c>
+      <c r="G106">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="107" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A107" t="s">
+        <v>53</v>
+      </c>
+      <c r="D107" t="s">
+        <v>24</v>
+      </c>
+      <c r="G107">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="108" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A108" t="s">
+        <v>53</v>
+      </c>
+      <c r="D108" t="s">
+        <v>25</v>
+      </c>
+      <c r="G108">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="109" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A109" t="s">
+        <v>53</v>
+      </c>
+      <c r="D109" t="s">
+        <v>26</v>
+      </c>
+      <c r="G109">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A110" t="s">
+        <v>54</v>
+      </c>
+      <c r="D110" t="s">
+        <v>24</v>
+      </c>
+      <c r="G110">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="111" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A111" t="s">
+        <v>54</v>
+      </c>
+      <c r="D111" t="s">
+        <v>25</v>
+      </c>
+      <c r="G111">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="112" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A112" t="s">
+        <v>54</v>
+      </c>
+      <c r="D112" t="s">
+        <v>26</v>
+      </c>
+      <c r="G112">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A113" t="s">
+        <v>55</v>
+      </c>
+      <c r="D113" t="s">
+        <v>24</v>
+      </c>
+      <c r="G113">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A114" t="s">
+        <v>55</v>
+      </c>
+      <c r="D114" t="s">
+        <v>25</v>
+      </c>
+      <c r="G114">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A115" t="s">
+        <v>55</v>
+      </c>
+      <c r="D115" t="s">
+        <v>26</v>
+      </c>
+      <c r="G115">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A116" t="s">
+        <v>56</v>
+      </c>
+      <c r="D116" t="s">
+        <v>24</v>
+      </c>
+      <c r="G116">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A117" t="s">
+        <v>56</v>
+      </c>
+      <c r="D117" t="s">
+        <v>25</v>
+      </c>
+      <c r="G117">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A118" t="s">
+        <v>56</v>
+      </c>
+      <c r="D118" t="s">
+        <v>26</v>
+      </c>
+      <c r="G118">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A119" t="s">
+        <v>57</v>
+      </c>
+      <c r="D119" t="s">
+        <v>24</v>
+      </c>
+      <c r="G119">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A120" t="s">
+        <v>57</v>
+      </c>
+      <c r="D120" t="s">
+        <v>25</v>
+      </c>
+      <c r="G120">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A121" t="s">
+        <v>57</v>
+      </c>
+      <c r="D121" t="s">
+        <v>26</v>
+      </c>
+      <c r="G121">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A122" t="s">
+        <v>58</v>
+      </c>
+      <c r="D122" t="s">
+        <v>24</v>
+      </c>
+      <c r="G122">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A123" t="s">
+        <v>58</v>
+      </c>
+      <c r="D123" t="s">
+        <v>25</v>
+      </c>
+      <c r="G123">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A124" t="s">
+        <v>58</v>
+      </c>
+      <c r="D124" t="s">
+        <v>26</v>
+      </c>
+      <c r="G124">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A125" t="s">
+        <v>59</v>
+      </c>
+      <c r="D125" t="s">
+        <v>24</v>
+      </c>
+      <c r="G125">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A126" t="s">
+        <v>59</v>
+      </c>
+      <c r="D126" t="s">
+        <v>25</v>
+      </c>
+      <c r="G126">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A127" t="s">
+        <v>59</v>
+      </c>
+      <c r="D127" t="s">
+        <v>26</v>
+      </c>
+      <c r="G127">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A128" t="s">
+        <v>60</v>
+      </c>
+      <c r="D128" t="s">
+        <v>24</v>
+      </c>
+      <c r="G128">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="129" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A129" t="s">
+        <v>60</v>
+      </c>
+      <c r="D129" t="s">
+        <v>25</v>
+      </c>
+      <c r="G129">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="130" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A130" t="s">
+        <v>60</v>
+      </c>
+      <c r="D130" t="s">
+        <v>26</v>
+      </c>
+      <c r="G130">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="131" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A131" t="s">
+        <v>61</v>
+      </c>
+      <c r="D131" t="s">
+        <v>24</v>
+      </c>
+      <c r="G131">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="132" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A132" t="s">
+        <v>61</v>
+      </c>
+      <c r="D132" t="s">
+        <v>25</v>
+      </c>
+      <c r="G132">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="133" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A133" t="s">
+        <v>61</v>
+      </c>
+      <c r="D133" t="s">
+        <v>26</v>
+      </c>
+      <c r="G133">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="134" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A134" t="s">
+        <v>62</v>
+      </c>
+      <c r="D134" t="s">
+        <v>24</v>
+      </c>
+      <c r="G134">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="135" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A135" t="s">
+        <v>62</v>
+      </c>
+      <c r="D135" t="s">
+        <v>25</v>
+      </c>
+      <c r="G135">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="136" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A136" t="s">
+        <v>62</v>
+      </c>
+      <c r="D136" t="s">
+        <v>26</v>
+      </c>
+      <c r="G136">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="137" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A137" t="s">
+        <v>63</v>
+      </c>
+      <c r="D137" t="s">
+        <v>24</v>
+      </c>
+      <c r="G137">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="138" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A138" t="s">
+        <v>63</v>
+      </c>
+      <c r="D138" t="s">
+        <v>25</v>
+      </c>
+      <c r="G138">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="139" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A139" t="s">
+        <v>63</v>
+      </c>
+      <c r="D139" t="s">
+        <v>26</v>
+      </c>
+      <c r="G139">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="140" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A140" t="s">
+        <v>48</v>
+      </c>
+      <c r="C140" t="s">
+        <v>111</v>
+      </c>
+      <c r="D140" t="s">
+        <v>51</v>
+      </c>
+      <c r="G140">
+        <v>100</v>
+      </c>
+      <c r="L140" t="s">
+        <v>112</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Sprint 4 coverage_report.xlsx updated info
</commit_message>
<xml_diff>
--- a/Evidence/MA/coverage_report.xlsx
+++ b/Evidence/MA/coverage_report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raygu\Downloads\CO3095\Evidence\MA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4471854-6991-423E-9D05-24281E973204}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE278C52-C0BF-42EB-A8BE-FE2379FDE6DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="16186" xr2:uid="{B4F26AE1-5879-47D9-8144-9A3C1A46093E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="142">
   <si>
     <t>Story ID</t>
   </si>
@@ -371,10 +371,97 @@
     <t xml:space="preserve">player_core, player_queue </t>
   </si>
   <si>
-    <t>Sprint 4 Total Coverate</t>
-  </si>
-  <si>
-    <t>All Code Modules</t>
+    <t>S4-01</t>
+  </si>
+  <si>
+    <t>S4-02</t>
+  </si>
+  <si>
+    <t>S4-03</t>
+  </si>
+  <si>
+    <t>S4-04</t>
+  </si>
+  <si>
+    <t>S4-05</t>
+  </si>
+  <si>
+    <t>S4-06</t>
+  </si>
+  <si>
+    <t>S4-07</t>
+  </si>
+  <si>
+    <t>S4-08</t>
+  </si>
+  <si>
+    <t>S4-09</t>
+  </si>
+  <si>
+    <t>S4-10</t>
+  </si>
+  <si>
+    <t>S4-11</t>
+  </si>
+  <si>
+    <t>S4-12</t>
+  </si>
+  <si>
+    <t>Sprint 4 Total Coverage</t>
+  </si>
+  <si>
+    <t>resume state</t>
+  </si>
+  <si>
+    <t>remember settings</t>
+  </si>
+  <si>
+    <t>schedule playback</t>
+  </si>
+  <si>
+    <t>import songs</t>
+  </si>
+  <si>
+    <t>custom tags</t>
+  </si>
+  <si>
+    <t>recently added</t>
+  </si>
+  <si>
+    <t>user profiles</t>
+  </si>
+  <si>
+    <t>playback stats</t>
+  </si>
+  <si>
+    <t>advanced search</t>
+  </si>
+  <si>
+    <t>export playlist</t>
+  </si>
+  <si>
+    <t>update metadata</t>
+  </si>
+  <si>
+    <t>rate songs</t>
+  </si>
+  <si>
+    <t>player_config</t>
+  </si>
+  <si>
+    <t>player_time</t>
+  </si>
+  <si>
+    <t>player_io</t>
+  </si>
+  <si>
+    <t>user_data</t>
+  </si>
+  <si>
+    <t>Overall Project Total Coverage</t>
+  </si>
+  <si>
+    <t>player_io, player_config, user_data, player_time</t>
   </si>
 </sst>
 </file>
@@ -762,7 +849,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6C833DE-F332-4BAA-A701-CCE6281E1DB6}">
-  <dimension ref="A1:L140"/>
+  <dimension ref="A1:L132"/>
   <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="3" max="3" width="29.52734375" customWidth="1"/>
@@ -4693,415 +4780,1104 @@
     </row>
     <row r="104" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A104" t="s">
-        <v>52</v>
+        <v>111</v>
+      </c>
+      <c r="B104">
+        <v>4</v>
+      </c>
+      <c r="C104" t="s">
+        <v>125</v>
       </c>
       <c r="D104" t="s">
         <v>24</v>
       </c>
+      <c r="E104">
+        <v>10</v>
+      </c>
+      <c r="F104">
+        <v>10</v>
+      </c>
       <c r="G104">
         <v>100</v>
+      </c>
+      <c r="H104">
+        <v>121</v>
+      </c>
+      <c r="I104">
+        <v>197</v>
+      </c>
+      <c r="J104">
+        <v>61</v>
+      </c>
+      <c r="K104" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L104" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="105" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A105" t="s">
-        <v>52</v>
+        <v>111</v>
+      </c>
+      <c r="B105">
+        <v>4</v>
+      </c>
+      <c r="C105" t="s">
+        <v>125</v>
       </c>
       <c r="D105" t="s">
         <v>25</v>
       </c>
+      <c r="E105">
+        <v>12</v>
+      </c>
+      <c r="F105">
+        <v>12</v>
+      </c>
       <c r="G105">
         <v>100</v>
+      </c>
+      <c r="H105">
+        <v>68</v>
+      </c>
+      <c r="I105">
+        <v>197</v>
+      </c>
+      <c r="J105">
+        <v>35</v>
+      </c>
+      <c r="K105" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L105" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="106" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A106" t="s">
-        <v>52</v>
+        <v>111</v>
+      </c>
+      <c r="B106">
+        <v>4</v>
+      </c>
+      <c r="C106" t="s">
+        <v>125</v>
       </c>
       <c r="D106" t="s">
         <v>26</v>
       </c>
+      <c r="E106">
+        <v>30</v>
+      </c>
+      <c r="F106">
+        <v>30</v>
+      </c>
       <c r="G106">
         <v>100</v>
+      </c>
+      <c r="H106">
+        <v>163</v>
+      </c>
+      <c r="I106">
+        <v>197</v>
+      </c>
+      <c r="J106">
+        <v>83</v>
+      </c>
+      <c r="K106" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L106" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A107" t="s">
-        <v>53</v>
+        <v>112</v>
+      </c>
+      <c r="B107">
+        <v>4</v>
+      </c>
+      <c r="C107" t="s">
+        <v>126</v>
       </c>
       <c r="D107" t="s">
         <v>24</v>
       </c>
+      <c r="E107">
+        <v>5</v>
+      </c>
+      <c r="F107">
+        <v>5</v>
+      </c>
       <c r="G107">
         <v>100</v>
+      </c>
+      <c r="H107">
+        <v>109</v>
+      </c>
+      <c r="I107">
+        <v>155</v>
+      </c>
+      <c r="J107">
+        <v>70</v>
+      </c>
+      <c r="K107" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L107" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A108" t="s">
-        <v>53</v>
+        <v>112</v>
+      </c>
+      <c r="B108">
+        <v>4</v>
+      </c>
+      <c r="C108" t="s">
+        <v>126</v>
       </c>
       <c r="D108" t="s">
         <v>25</v>
       </c>
+      <c r="E108">
+        <v>23</v>
+      </c>
+      <c r="F108">
+        <v>23</v>
+      </c>
       <c r="G108">
         <v>100</v>
+      </c>
+      <c r="H108">
+        <v>43</v>
+      </c>
+      <c r="I108">
+        <v>155</v>
+      </c>
+      <c r="J108">
+        <v>28</v>
+      </c>
+      <c r="K108" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L108" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A109" t="s">
-        <v>53</v>
+        <v>112</v>
+      </c>
+      <c r="B109">
+        <v>4</v>
+      </c>
+      <c r="C109" t="s">
+        <v>126</v>
       </c>
       <c r="D109" t="s">
         <v>26</v>
       </c>
+      <c r="E109">
+        <v>6</v>
+      </c>
+      <c r="F109">
+        <v>6</v>
+      </c>
       <c r="G109">
         <v>100</v>
+      </c>
+      <c r="H109">
+        <v>52</v>
+      </c>
+      <c r="I109">
+        <v>155</v>
+      </c>
+      <c r="J109">
+        <v>34</v>
+      </c>
+      <c r="K109" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L109" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="110" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A110" t="s">
-        <v>54</v>
+        <v>113</v>
+      </c>
+      <c r="B110">
+        <v>4</v>
+      </c>
+      <c r="C110" t="s">
+        <v>124</v>
       </c>
       <c r="D110" t="s">
         <v>24</v>
       </c>
+      <c r="E110">
+        <v>5</v>
+      </c>
+      <c r="F110">
+        <v>5</v>
+      </c>
       <c r="G110">
         <v>100</v>
+      </c>
+      <c r="H110">
+        <v>109</v>
+      </c>
+      <c r="I110">
+        <v>155</v>
+      </c>
+      <c r="J110">
+        <v>70</v>
+      </c>
+      <c r="K110" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L110" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="111" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A111" t="s">
-        <v>54</v>
+        <v>113</v>
+      </c>
+      <c r="B111">
+        <v>4</v>
+      </c>
+      <c r="C111" t="s">
+        <v>124</v>
       </c>
       <c r="D111" t="s">
         <v>25</v>
       </c>
+      <c r="E111">
+        <v>23</v>
+      </c>
+      <c r="F111">
+        <v>23</v>
+      </c>
       <c r="G111">
         <v>100</v>
+      </c>
+      <c r="H111">
+        <v>43</v>
+      </c>
+      <c r="I111">
+        <v>155</v>
+      </c>
+      <c r="J111">
+        <v>28</v>
+      </c>
+      <c r="K111" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L111" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="112" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A112" t="s">
-        <v>54</v>
+        <v>113</v>
+      </c>
+      <c r="B112">
+        <v>4</v>
+      </c>
+      <c r="C112" t="s">
+        <v>124</v>
       </c>
       <c r="D112" t="s">
         <v>26</v>
       </c>
+      <c r="E112">
+        <v>6</v>
+      </c>
+      <c r="F112">
+        <v>6</v>
+      </c>
       <c r="G112">
         <v>100</v>
       </c>
-    </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="H112">
+        <v>52</v>
+      </c>
+      <c r="I112">
+        <v>155</v>
+      </c>
+      <c r="J112">
+        <v>34</v>
+      </c>
+      <c r="K112" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L112" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="113" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A113" t="s">
-        <v>55</v>
+        <v>114</v>
+      </c>
+      <c r="B113">
+        <v>4</v>
+      </c>
+      <c r="C113" t="s">
+        <v>127</v>
       </c>
       <c r="D113" t="s">
         <v>24</v>
       </c>
+      <c r="E113">
+        <v>11</v>
+      </c>
+      <c r="F113">
+        <v>11</v>
+      </c>
       <c r="G113">
         <v>100</v>
       </c>
-    </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="H113">
+        <v>55</v>
+      </c>
+      <c r="I113">
+        <v>121</v>
+      </c>
+      <c r="J113">
+        <v>45</v>
+      </c>
+      <c r="K113" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L113" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="114" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A114" t="s">
-        <v>55</v>
+        <v>115</v>
+      </c>
+      <c r="B114">
+        <v>4</v>
+      </c>
+      <c r="C114" t="s">
+        <v>128</v>
       </c>
       <c r="D114" t="s">
+        <v>24</v>
+      </c>
+      <c r="E114">
+        <v>10</v>
+      </c>
+      <c r="F114">
+        <v>10</v>
+      </c>
+      <c r="G114">
+        <v>100</v>
+      </c>
+      <c r="H114">
+        <v>121</v>
+      </c>
+      <c r="I114">
+        <v>197</v>
+      </c>
+      <c r="J114">
+        <v>61</v>
+      </c>
+      <c r="K114" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L114" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="115" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A115" t="s">
+        <v>115</v>
+      </c>
+      <c r="B115">
+        <v>4</v>
+      </c>
+      <c r="C115" t="s">
+        <v>128</v>
+      </c>
+      <c r="D115" t="s">
         <v>25</v>
       </c>
-      <c r="G114">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A115" t="s">
-        <v>55</v>
-      </c>
-      <c r="D115" t="s">
+      <c r="E115">
+        <v>12</v>
+      </c>
+      <c r="F115">
+        <v>12</v>
+      </c>
+      <c r="G115">
+        <v>100</v>
+      </c>
+      <c r="H115">
+        <v>68</v>
+      </c>
+      <c r="I115">
+        <v>197</v>
+      </c>
+      <c r="J115">
+        <v>35</v>
+      </c>
+      <c r="K115" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L115" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="116" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A116" t="s">
+        <v>115</v>
+      </c>
+      <c r="B116">
+        <v>4</v>
+      </c>
+      <c r="C116" t="s">
+        <v>128</v>
+      </c>
+      <c r="D116" t="s">
         <v>26</v>
       </c>
-      <c r="G115">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A116" t="s">
-        <v>56</v>
-      </c>
-      <c r="D116" t="s">
+      <c r="E116">
+        <v>30</v>
+      </c>
+      <c r="F116">
+        <v>30</v>
+      </c>
+      <c r="G116">
+        <v>100</v>
+      </c>
+      <c r="H116">
+        <v>163</v>
+      </c>
+      <c r="I116">
+        <v>197</v>
+      </c>
+      <c r="J116">
+        <v>83</v>
+      </c>
+      <c r="K116" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L116" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="117" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A117" t="s">
+        <v>116</v>
+      </c>
+      <c r="B117">
+        <v>4</v>
+      </c>
+      <c r="C117" t="s">
+        <v>129</v>
+      </c>
+      <c r="D117" t="s">
         <v>24</v>
       </c>
-      <c r="G116">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A117" t="s">
-        <v>56</v>
-      </c>
-      <c r="D117" t="s">
+      <c r="E117">
+        <v>5</v>
+      </c>
+      <c r="F117">
+        <v>5</v>
+      </c>
+      <c r="G117">
+        <v>100</v>
+      </c>
+      <c r="H117">
+        <v>109</v>
+      </c>
+      <c r="I117">
+        <v>155</v>
+      </c>
+      <c r="J117">
+        <v>70</v>
+      </c>
+      <c r="K117" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L117" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="118" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A118" t="s">
+        <v>116</v>
+      </c>
+      <c r="B118">
+        <v>4</v>
+      </c>
+      <c r="C118" t="s">
+        <v>129</v>
+      </c>
+      <c r="D118" t="s">
         <v>25</v>
       </c>
-      <c r="G117">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A118" t="s">
-        <v>56</v>
-      </c>
-      <c r="D118" t="s">
+      <c r="E118">
+        <v>23</v>
+      </c>
+      <c r="F118">
+        <v>23</v>
+      </c>
+      <c r="G118">
+        <v>100</v>
+      </c>
+      <c r="H118">
+        <v>43</v>
+      </c>
+      <c r="I118">
+        <v>155</v>
+      </c>
+      <c r="J118">
+        <v>28</v>
+      </c>
+      <c r="K118" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L118" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="119" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A119" t="s">
+        <v>116</v>
+      </c>
+      <c r="B119">
+        <v>4</v>
+      </c>
+      <c r="C119" t="s">
+        <v>129</v>
+      </c>
+      <c r="D119" t="s">
         <v>26</v>
       </c>
-      <c r="G118">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A119" t="s">
-        <v>57</v>
-      </c>
-      <c r="D119" t="s">
-        <v>24</v>
+      <c r="E119">
+        <v>6</v>
+      </c>
+      <c r="F119">
+        <v>6</v>
       </c>
       <c r="G119">
         <v>100</v>
       </c>
-    </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="H119">
+        <v>52</v>
+      </c>
+      <c r="I119">
+        <v>155</v>
+      </c>
+      <c r="J119">
+        <v>34</v>
+      </c>
+      <c r="K119" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L119" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="120" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A120" t="s">
-        <v>57</v>
+        <v>117</v>
+      </c>
+      <c r="B120">
+        <v>4</v>
+      </c>
+      <c r="C120" t="s">
+        <v>130</v>
       </c>
       <c r="D120" t="s">
         <v>25</v>
       </c>
+      <c r="E120">
+        <v>25</v>
+      </c>
+      <c r="F120">
+        <v>25</v>
+      </c>
       <c r="G120">
         <v>100</v>
       </c>
-    </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="H120">
+        <v>87</v>
+      </c>
+      <c r="I120">
+        <v>222</v>
+      </c>
+      <c r="J120">
+        <v>39</v>
+      </c>
+      <c r="K120" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L120" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="121" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A121" t="s">
-        <v>57</v>
+        <v>117</v>
+      </c>
+      <c r="B121">
+        <v>4</v>
+      </c>
+      <c r="C121" t="s">
+        <v>130</v>
       </c>
       <c r="D121" t="s">
         <v>26</v>
       </c>
+      <c r="E121">
+        <v>17</v>
+      </c>
+      <c r="F121">
+        <v>17</v>
+      </c>
       <c r="G121">
         <v>100</v>
       </c>
-    </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="H121">
+        <v>140</v>
+      </c>
+      <c r="I121">
+        <v>222</v>
+      </c>
+      <c r="J121">
+        <v>63</v>
+      </c>
+      <c r="K121" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L121" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="122" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A122" t="s">
-        <v>58</v>
+        <v>118</v>
+      </c>
+      <c r="B122">
+        <v>4</v>
+      </c>
+      <c r="C122" t="s">
+        <v>131</v>
       </c>
       <c r="D122" t="s">
         <v>24</v>
       </c>
+      <c r="E122">
+        <v>10</v>
+      </c>
+      <c r="F122">
+        <v>10</v>
+      </c>
       <c r="G122">
         <v>100</v>
       </c>
-    </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="H122">
+        <v>121</v>
+      </c>
+      <c r="I122">
+        <v>197</v>
+      </c>
+      <c r="J122">
+        <v>61</v>
+      </c>
+      <c r="K122" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L122" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="123" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A123" t="s">
-        <v>58</v>
+        <v>118</v>
+      </c>
+      <c r="B123">
+        <v>4</v>
+      </c>
+      <c r="C123" t="s">
+        <v>131</v>
       </c>
       <c r="D123" t="s">
         <v>25</v>
       </c>
+      <c r="E123">
+        <v>12</v>
+      </c>
+      <c r="F123">
+        <v>12</v>
+      </c>
       <c r="G123">
         <v>100</v>
       </c>
-    </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="H123">
+        <v>68</v>
+      </c>
+      <c r="I123">
+        <v>197</v>
+      </c>
+      <c r="J123">
+        <v>35</v>
+      </c>
+      <c r="K123" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L123" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="124" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A124" t="s">
-        <v>58</v>
+        <v>118</v>
+      </c>
+      <c r="B124">
+        <v>4</v>
+      </c>
+      <c r="C124" t="s">
+        <v>131</v>
       </c>
       <c r="D124" t="s">
         <v>26</v>
       </c>
+      <c r="E124">
+        <v>30</v>
+      </c>
+      <c r="F124">
+        <v>30</v>
+      </c>
       <c r="G124">
         <v>100</v>
       </c>
-    </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="H124">
+        <v>163</v>
+      </c>
+      <c r="I124">
+        <v>197</v>
+      </c>
+      <c r="J124">
+        <v>83</v>
+      </c>
+      <c r="K124" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L124" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="125" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A125" t="s">
-        <v>59</v>
+        <v>119</v>
+      </c>
+      <c r="B125">
+        <v>4</v>
+      </c>
+      <c r="C125" t="s">
+        <v>132</v>
       </c>
       <c r="D125" t="s">
+        <v>25</v>
+      </c>
+      <c r="E125">
+        <v>25</v>
+      </c>
+      <c r="F125">
+        <v>25</v>
+      </c>
+      <c r="G125">
+        <v>100</v>
+      </c>
+      <c r="H125">
+        <v>87</v>
+      </c>
+      <c r="I125">
+        <v>222</v>
+      </c>
+      <c r="J125">
+        <v>39</v>
+      </c>
+      <c r="K125" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L125" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="126" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A126" t="s">
+        <v>119</v>
+      </c>
+      <c r="B126">
+        <v>4</v>
+      </c>
+      <c r="C126" t="s">
+        <v>132</v>
+      </c>
+      <c r="D126" t="s">
+        <v>26</v>
+      </c>
+      <c r="E126">
+        <v>17</v>
+      </c>
+      <c r="F126">
+        <v>17</v>
+      </c>
+      <c r="G126">
+        <v>100</v>
+      </c>
+      <c r="H126">
+        <v>140</v>
+      </c>
+      <c r="I126">
+        <v>222</v>
+      </c>
+      <c r="J126">
+        <v>63</v>
+      </c>
+      <c r="K126" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L126" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="127" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A127" t="s">
+        <v>120</v>
+      </c>
+      <c r="B127">
+        <v>4</v>
+      </c>
+      <c r="C127" t="s">
+        <v>133</v>
+      </c>
+      <c r="D127" t="s">
         <v>24</v>
       </c>
-      <c r="G125">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A126" t="s">
-        <v>59</v>
-      </c>
-      <c r="D126" t="s">
-        <v>25</v>
-      </c>
-      <c r="G126">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.5">
-      <c r="A127" t="s">
-        <v>59</v>
-      </c>
-      <c r="D127" t="s">
-        <v>26</v>
+      <c r="E127">
+        <v>11</v>
+      </c>
+      <c r="F127">
+        <v>11</v>
       </c>
       <c r="G127">
         <v>100</v>
       </c>
-    </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="H127">
+        <v>55</v>
+      </c>
+      <c r="I127">
+        <v>121</v>
+      </c>
+      <c r="J127">
+        <v>45</v>
+      </c>
+      <c r="K127" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L127" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="128" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A128" t="s">
-        <v>60</v>
+        <v>121</v>
+      </c>
+      <c r="B128">
+        <v>4</v>
+      </c>
+      <c r="C128" t="s">
+        <v>134</v>
       </c>
       <c r="D128" t="s">
         <v>24</v>
       </c>
+      <c r="E128">
+        <v>11</v>
+      </c>
+      <c r="F128">
+        <v>11</v>
+      </c>
       <c r="G128">
         <v>100</v>
+      </c>
+      <c r="H128">
+        <v>55</v>
+      </c>
+      <c r="I128">
+        <v>121</v>
+      </c>
+      <c r="J128">
+        <v>45</v>
+      </c>
+      <c r="K128" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L128" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="129" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A129" t="s">
-        <v>60</v>
+        <v>122</v>
+      </c>
+      <c r="B129">
+        <v>4</v>
+      </c>
+      <c r="C129" t="s">
+        <v>135</v>
       </c>
       <c r="D129" t="s">
         <v>25</v>
       </c>
+      <c r="E129">
+        <v>25</v>
+      </c>
+      <c r="F129">
+        <v>25</v>
+      </c>
       <c r="G129">
         <v>100</v>
+      </c>
+      <c r="H129">
+        <v>87</v>
+      </c>
+      <c r="I129">
+        <v>222</v>
+      </c>
+      <c r="J129">
+        <v>39</v>
+      </c>
+      <c r="K129" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L129" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="130" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A130" t="s">
-        <v>60</v>
+        <v>122</v>
+      </c>
+      <c r="B130">
+        <v>4</v>
+      </c>
+      <c r="C130" t="s">
+        <v>135</v>
       </c>
       <c r="D130" t="s">
         <v>26</v>
       </c>
+      <c r="E130">
+        <v>17</v>
+      </c>
+      <c r="F130">
+        <v>17</v>
+      </c>
       <c r="G130">
         <v>100</v>
+      </c>
+      <c r="H130">
+        <v>140</v>
+      </c>
+      <c r="I130">
+        <v>222</v>
+      </c>
+      <c r="J130">
+        <v>63</v>
+      </c>
+      <c r="K130" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L130" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="131" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A131" t="s">
-        <v>61</v>
+        <v>48</v>
+      </c>
+      <c r="B131">
+        <v>4</v>
+      </c>
+      <c r="C131" t="s">
+        <v>123</v>
       </c>
       <c r="D131" t="s">
-        <v>24</v>
+        <v>51</v>
+      </c>
+      <c r="E131">
+        <v>139</v>
+      </c>
+      <c r="F131">
+        <v>139</v>
       </c>
       <c r="G131">
         <v>100</v>
+      </c>
+      <c r="H131">
+        <v>503</v>
+      </c>
+      <c r="I131">
+        <v>695</v>
+      </c>
+      <c r="J131">
+        <v>72</v>
+      </c>
+      <c r="K131" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L131" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="132" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A132" t="s">
-        <v>61</v>
+        <v>48</v>
+      </c>
+      <c r="B132">
+        <v>4</v>
+      </c>
+      <c r="C132" t="s">
+        <v>140</v>
       </c>
       <c r="D132" t="s">
-        <v>25</v>
+        <v>51</v>
+      </c>
+      <c r="E132">
+        <v>627</v>
+      </c>
+      <c r="F132">
+        <v>627</v>
       </c>
       <c r="G132">
         <v>100</v>
       </c>
-    </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A133" t="s">
-        <v>61</v>
-      </c>
-      <c r="D133" t="s">
-        <v>26</v>
-      </c>
-      <c r="G133">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A134" t="s">
-        <v>62</v>
-      </c>
-      <c r="D134" t="s">
-        <v>24</v>
-      </c>
-      <c r="G134">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A135" t="s">
-        <v>62</v>
-      </c>
-      <c r="D135" t="s">
-        <v>25</v>
-      </c>
-      <c r="G135">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A136" t="s">
-        <v>62</v>
-      </c>
-      <c r="D136" t="s">
-        <v>26</v>
-      </c>
-      <c r="G136">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A137" t="s">
-        <v>63</v>
-      </c>
-      <c r="D137" t="s">
-        <v>24</v>
-      </c>
-      <c r="G137">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A138" t="s">
-        <v>63</v>
-      </c>
-      <c r="D138" t="s">
-        <v>25</v>
-      </c>
-      <c r="G138">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A139" t="s">
-        <v>63</v>
-      </c>
-      <c r="D139" t="s">
-        <v>26</v>
-      </c>
-      <c r="G139">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A140" t="s">
-        <v>48</v>
-      </c>
-      <c r="C140" t="s">
-        <v>111</v>
-      </c>
-      <c r="D140" t="s">
+      <c r="H132">
+        <v>2625</v>
+      </c>
+      <c r="I132">
+        <v>3119</v>
+      </c>
+      <c r="J132">
+        <v>84</v>
+      </c>
+      <c r="K132" s="2">
+        <v>46025</v>
+      </c>
+      <c r="L132" t="s">
         <v>51</v>
-      </c>
-      <c r="G140">
-        <v>100</v>
-      </c>
-      <c r="L140" t="s">
-        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>